<commit_message>
Publish September 14–20 substitutions and transfers
</commit_message>
<xml_diff>
--- a/InformacjeOZastepstwach.xlsx
+++ b/InformacjeOZastepstwach.xlsx
@@ -9,511 +9,396 @@
   <sheets>
     <sheet name="Opis parametrów" sheetId="2" r:id="rId2"/>
     <sheet name="Oddziały" sheetId="3" r:id="rId3"/>
-    <sheet name="Dyżury" sheetId="4" r:id="rId4"/>
+    <sheet name="Dzienniki zajeć innych" sheetId="4" r:id="rId4"/>
+    <sheet name="Dyżury" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Oddziały!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Dyżury!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dzienniki zajeć innych'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Dyżury!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="164">
-  <si>
-    <t>Rok szkolny: 2026/2027</t>
-  </si>
-  <si>
-    <t>Okres: 07.09.2026 (pon.) - 13.09.2026 (niedz.)</t>
-  </si>
-  <si>
-    <t>Dzień</t>
-  </si>
-  <si>
-    <t>Lekcja</t>
-  </si>
-  <si>
-    <t>Nauczyciel/wakat</t>
-  </si>
-  <si>
-    <t>Oddział</t>
-  </si>
-  <si>
-    <t>Przedmiot</t>
-  </si>
-  <si>
-    <t>Sala</t>
-  </si>
-  <si>
-    <t>Zastępca</t>
-  </si>
-  <si>
-    <t>Uwagi</t>
-  </si>
-  <si>
-    <t>Forma płatności</t>
-  </si>
-  <si>
-    <t>07.09.2026</t>
-  </si>
-  <si>
-    <t>1, 08:00-08:45</t>
-  </si>
-  <si>
-    <t>Stępień Krystyna</t>
-  </si>
-  <si>
-    <t>2CA</t>
-  </si>
-  <si>
-    <t>Technika w produkcji cukierniczej</t>
-  </si>
-  <si>
-    <t>prs</t>
-  </si>
-  <si>
-    <t>Uczniowie przychodzą później</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>2, 08:50-09:35</t>
-  </si>
-  <si>
-    <t>3, 09:40-10:25</t>
-  </si>
-  <si>
-    <t>3CA</t>
-  </si>
-  <si>
-    <t>4, 10:35-11:20</t>
-  </si>
-  <si>
-    <t>Sobczak Anna</t>
-  </si>
-  <si>
-    <t>2FA</t>
-  </si>
-  <si>
-    <t>Język angielski</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Biezmienow Małgorzata</t>
-  </si>
-  <si>
-    <t>Dodatkowo płatne</t>
-  </si>
-  <si>
-    <t>Technologie produkcji cukierniczej</t>
-  </si>
-  <si>
-    <t>5, 11:25-12:10</t>
-  </si>
-  <si>
-    <t>Najwer Maciej</t>
-  </si>
-  <si>
-    <t>1TFA|gr1</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>Granatowska Mariola</t>
-  </si>
-  <si>
-    <t>Zajęcia biblioteczne</t>
-  </si>
-  <si>
-    <t>bib</t>
-  </si>
-  <si>
-    <t>Wrzeszcz Barbara</t>
-  </si>
-  <si>
-    <t>Bezpłatne</t>
-  </si>
-  <si>
-    <t>1CA</t>
-  </si>
-  <si>
-    <t>Historia</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>Kaczorowski Waldemar</t>
-  </si>
-  <si>
-    <t>6, 12:25-13:10</t>
-  </si>
-  <si>
-    <t>1TFH|gr2</t>
-  </si>
-  <si>
-    <t>1FB</t>
-  </si>
-  <si>
-    <t>Techniki fryzjerskie</t>
-  </si>
-  <si>
-    <t>prF3</t>
-  </si>
-  <si>
-    <t>Uczniowie zwolnieni do domu</t>
-  </si>
-  <si>
-    <t>Zajęcia z wychowawcą</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>Galert Anna</t>
-  </si>
-  <si>
-    <t>7, 13:15-14:00</t>
-  </si>
-  <si>
-    <t>8, 14:05-14:50</t>
-  </si>
-  <si>
-    <t>Filusz Marzena</t>
-  </si>
-  <si>
-    <t>4TFB</t>
-  </si>
-  <si>
-    <t>Rozwój kompetencji zawodowych - matematyka w działalności gospodarczej</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>1TFB|gr1</t>
-  </si>
-  <si>
-    <t>Zając Ewa</t>
-  </si>
-  <si>
-    <t>9, 14:55-15:40</t>
-  </si>
-  <si>
-    <t>4TFA</t>
-  </si>
-  <si>
-    <t>Matematyka</t>
-  </si>
-  <si>
-    <t>Filipiak Wiesław</t>
-  </si>
-  <si>
-    <t>11, 16:35-17:20</t>
-  </si>
-  <si>
-    <t>Krystek Krzysztof</t>
-  </si>
-  <si>
-    <t>1B</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>12, 17:25-18:10</t>
-  </si>
-  <si>
-    <t>13, 18:15-19:00</t>
-  </si>
-  <si>
-    <t>08.09.2026</t>
-  </si>
-  <si>
-    <t>1TFB|gr2</t>
-  </si>
-  <si>
-    <t>Zajęcia praktyczne - wykonywanie usług fryzjerskich</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>Jaworska Edyta</t>
-  </si>
-  <si>
-    <t>prf2</t>
-  </si>
-  <si>
-    <t>Leńczowska Iwona</t>
-  </si>
-  <si>
-    <t>10, 15:45-16:30</t>
-  </si>
-  <si>
-    <t>2TFB</t>
-  </si>
-  <si>
-    <t>09.09.2026</t>
-  </si>
-  <si>
-    <t>Krycia Ewelina</t>
-  </si>
-  <si>
-    <t>Język polski</t>
-  </si>
-  <si>
-    <t>Informatyka</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>1CB</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>Zaleska Magdalena</t>
-  </si>
-  <si>
-    <t>1S</t>
-  </si>
-  <si>
-    <t>Biologia</t>
-  </si>
-  <si>
-    <t>Mucha Anna</t>
-  </si>
-  <si>
-    <t>2TFA</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>Kruk Marcin</t>
-  </si>
-  <si>
-    <t>3TFB|gr2</t>
-  </si>
-  <si>
-    <t>10.09.2026</t>
-  </si>
-  <si>
-    <t>1CB|fryzjer</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Jastrzębska-Majtyka Agnieszka</t>
-  </si>
-  <si>
-    <t>Kończyńska Małgorzata</t>
-  </si>
-  <si>
-    <t>5TFB</t>
-  </si>
-  <si>
-    <t>2CA|CH</t>
-  </si>
-  <si>
-    <t>Wychowanie fizyczne</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>Pietrycha Małgorzata</t>
-  </si>
-  <si>
-    <t>2CA|DZ</t>
-  </si>
-  <si>
-    <t>1FA|gr1</t>
-  </si>
-  <si>
-    <t>1FA|gr2</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>2WA</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>Wójcik Kamil</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>1FA</t>
-  </si>
-  <si>
-    <t>Filipek Anna</t>
-  </si>
-  <si>
-    <t>1TFB</t>
-  </si>
-  <si>
-    <t>Danielewski Paweł</t>
-  </si>
-  <si>
-    <t>Chemia</t>
-  </si>
-  <si>
-    <t>Ostrowska Ewa</t>
-  </si>
-  <si>
-    <t>2CB</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>1K</t>
-  </si>
-  <si>
-    <t>11.09.2026</t>
-  </si>
-  <si>
-    <t>Rozwój kompetencji zawodowych - dekoracje w cukiernictwie</t>
-  </si>
-  <si>
-    <t>Hudziec Agnieszka</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>Małecka Barbara</t>
-  </si>
-  <si>
-    <t>1TH</t>
-  </si>
-  <si>
-    <t>1TFA</t>
-  </si>
-  <si>
-    <t>Sałdyka Karolina</t>
-  </si>
-  <si>
-    <t>3FB</t>
-  </si>
-  <si>
-    <t>1TFH</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>Doradztwo zawodowe</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>Krzemińska Beata</t>
-  </si>
-  <si>
-    <t>Godzina</t>
-  </si>
-  <si>
-    <t>Nauczyciel</t>
-  </si>
-  <si>
-    <t>Miejsce dyżuru</t>
-  </si>
-  <si>
-    <t>10:25-10:35</t>
-  </si>
-  <si>
-    <t>boisko - dziedziniec wejściowy/boisko</t>
-  </si>
-  <si>
-    <t>Nowak Magdalena</t>
-  </si>
-  <si>
-    <t>13:10-13:15</t>
-  </si>
-  <si>
-    <t>14:00-14:05</t>
-  </si>
-  <si>
-    <t>14:50-14:55</t>
-  </si>
-  <si>
-    <t>piętro_1</t>
-  </si>
-  <si>
-    <t>Ulanowska Magdalena</t>
-  </si>
-  <si>
-    <t>16:30-16:35</t>
-  </si>
-  <si>
-    <t>Smereka Alicja</t>
-  </si>
-  <si>
-    <t>09:35-09:40</t>
-  </si>
-  <si>
-    <t>piętro_3</t>
-  </si>
-  <si>
-    <t>07:55-08:00</t>
-  </si>
-  <si>
-    <t>parter</t>
-  </si>
-  <si>
-    <t>11:20-11:25</t>
-  </si>
-  <si>
-    <t>Marzec Renata</t>
-  </si>
-  <si>
-    <t>12:10-12:25</t>
-  </si>
-  <si>
-    <t>Piątek-Pawłowska Bożena</t>
-  </si>
-  <si>
-    <t>piętro_2</t>
-  </si>
-  <si>
-    <t>Świerzewicz Katarzyna</t>
-  </si>
-  <si>
-    <t>Karczmarz Aleksandra</t>
-  </si>
-  <si>
-    <t>Biczysko Wojciech</t>
-  </si>
-  <si>
-    <t>Misiąg Anna</t>
-  </si>
-  <si>
-    <t>Kopij Marcin</t>
-  </si>
-  <si>
-    <t>15:40-15:45</t>
-  </si>
-</sst>
+<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="125">
+  <ns0:si>
+    <ns0:t>Rok szkolny: 2026/2027</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Okres: 14.09.2026 (pon.) - 20.09.2026 (niedz.)</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Dzień</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Lekcja</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Nauczyciel/wakat</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Oddział</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Przedmiot</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Sala</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Zastępca</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Uwagi</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Forma płatności</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>14.09.2026</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1, 08:00-08:45</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Stępień Krystyna</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2CA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Technika w produkcji cukierniczej</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>prs</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Kończyńska Małgorzata</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t/>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Dodatkowo płatne</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2, 08:50-09:35</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Krycia Ewelina</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1TFA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Biologia</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>31</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Sałdyka Karolina</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>3, 09:40-10:25</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Język polski</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>33</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Zastępstwo</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>-</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>3CA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>4, 10:35-11:20</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>3WA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Zajęcia biblioteczne</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>bib</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Wrzeszcz Barbara</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Bezpłatne</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Technologie produkcji cukierniczej</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>5, 11:25-12:10</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1FB</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Historia</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>18</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Kaczorowski Waldemar</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1CA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>6, 12:25-13:10</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2TFB</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>7, 13:15-14:00</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Zajęcia z wychowawcą</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Galert Anna</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>8, 14:05-14:50</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Filusz Marzena</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>4TFB</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Rozwój kompetencji zawodowych - matematyka w działalności gospodarczej</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>17</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Uczniowie zwolnieni do domu</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>9, 14:55-15:40</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>4TFA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Doradztwo zawodowe</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>5</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Krzemińska Beata</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>15.09.2026</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Jaworska Edyta</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1TFB|gr1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Zajęcia praktyczne - wykonywanie usług fryzjerskich</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>6</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Bez konsekwencji (nieobecny oddział nauczyciela)</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Sobczak Anna</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1TFB|gr2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>prf2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Misiąg Anna</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2WA|gr1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Język niemiecki</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>44</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2TFA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>3TFB|gr1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1TFA|gr1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1TFH|gr1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2TH</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Techniki fryzjerskie</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>10, 15:45-16:30</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>16.09.2026</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1CB</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1S</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Matematyka</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>17.09.2026</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Rozwój kompetencji zawodowych - dekoracje w cukiernictwie</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>5TFB</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1FA</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>18.09.2026</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Świerzewicz Katarzyna</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2K</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Technologia gastronomiczna z towaroznawstwem</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>29</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Okienko dla uczniów</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Godzina</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Nauczyciel</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Dziennik zajęć innych</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Opis zajęć</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>08:00-08:45</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t/>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>08:00-14:40</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Bokuniewicz Sylwia</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t/>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>dyżur pedagoga</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>08:50-09:35</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Miejsce dyżuru</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>08:45-08:50</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>piętro_3</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Kosin Anna</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>09:35-09:40</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>piętro_2</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>10:25-10:35</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>boisko - dziedziniec wejściowy/boisko</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Jastrzębska-Majtyka Agnieszka</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>07:55-08:00</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>parter</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>13:10-13:15</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>14:00-14:05</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>14:50-14:55</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>piętro_1</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>16:30-16:35</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>11:20-11:25</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>12:10-12:25</ns0:t>
+  </ns0:si>
+</ns0:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -961,7 +846,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{7b69b720-263f-409a-8ace-71751a1182b4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{07798d68-ff35-4714-beca-c4f6135787b9}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -982,17 +867,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{65802c7f-f101-4504-9092-87d613bbd669}">
-  <dimension ref="A1:I94"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{df400fe4-3e65-42b8-b0b6-7605c1b5066c}">
+  <dimension ref="A1:I78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
     <col min="2" max="2" width="14.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="19.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="11.2857142857143" customWidth="1"/>
+    <col min="3" max="3" width="21.1428571428571" customWidth="1"/>
+    <col min="4" max="4" width="10.5714285714286" customWidth="1"/>
     <col min="5" max="5" width="68.4285714285714" customWidth="1"/>
     <col min="6" max="6" width="7.42857142857143" customWidth="1"/>
-    <col min="7" max="7" width="28.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="45.5714285714286" customWidth="1"/>
     <col min="8" max="8" width="9.28571428571429" customWidth="1"/>
     <col min="9" max="9" width="17.8571428571429" customWidth="1"/>
   </cols>
@@ -1063,19 +948,19 @@
         <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H3" t="s">
         <v>18</v>
@@ -1089,13 +974,13 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
         <v>15</v>
@@ -1118,28 +1003,28 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H5" t="s">
         <v>18</v>
       </c>
       <c r="I5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15">
@@ -1147,16 +1032,16 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F6" t="s">
         <v>16</v>
@@ -1176,28 +1061,28 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H7" t="s">
         <v>18</v>
       </c>
       <c r="I7" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15">
@@ -1205,28 +1090,28 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
         <v>31</v>
       </c>
-      <c r="C8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" t="s">
-        <v>25</v>
-      </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="G8" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="H8" t="s">
         <v>18</v>
       </c>
       <c r="I8" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15">
@@ -1234,10 +1119,10 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
         <v>40</v>
@@ -1255,7 +1140,7 @@
         <v>18</v>
       </c>
       <c r="I9" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15">
@@ -1263,28 +1148,28 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" t="s">
         <v>44</v>
       </c>
-      <c r="C10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>45</v>
-      </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="F10" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="H10" t="s">
         <v>18</v>
       </c>
       <c r="I10" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15">
@@ -1292,28 +1177,28 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
         <v>46</v>
       </c>
       <c r="E11" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G11" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="H11" t="s">
         <v>18</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15">
@@ -1321,28 +1206,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
         <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F12" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="G12" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="H12" t="s">
         <v>18</v>
       </c>
       <c r="I12" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15">
@@ -1350,19 +1235,19 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G13" t="s">
         <v>49</v>
@@ -1379,28 +1264,28 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" t="s">
+        <v>52</v>
+      </c>
+      <c r="E14" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" t="s">
         <v>54</v>
       </c>
-      <c r="C14" t="s">
+      <c r="G14" t="s">
         <v>55</v>
       </c>
-      <c r="D14" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" t="s">
-        <v>57</v>
-      </c>
-      <c r="F14" t="s">
-        <v>58</v>
-      </c>
-      <c r="G14" t="s">
-        <v>49</v>
-      </c>
       <c r="H14" t="s">
         <v>18</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15">
@@ -1408,19 +1293,19 @@
         <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="D15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" t="s">
         <v>59</v>
-      </c>
-      <c r="E15" t="s">
-        <v>36</v>
-      </c>
-      <c r="F15" t="s">
-        <v>37</v>
       </c>
       <c r="G15" t="s">
         <v>60</v>
@@ -1429,1088 +1314,1088 @@
         <v>18</v>
       </c>
       <c r="I15" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H16" t="s">
         <v>18</v>
       </c>
       <c r="I16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" t="s">
+        <v>64</v>
+      </c>
+      <c r="F17" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" t="s">
         <v>66</v>
       </c>
-      <c r="D17" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" t="s">
-        <v>63</v>
-      </c>
-      <c r="F17" t="s">
-        <v>68</v>
-      </c>
-      <c r="G17" t="s">
-        <v>64</v>
-      </c>
       <c r="H17" t="s">
         <v>18</v>
       </c>
       <c r="I17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="C18" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F18" t="s">
+        <v>65</v>
+      </c>
+      <c r="G18" t="s">
         <v>66</v>
       </c>
-      <c r="D18" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" t="s">
-        <v>63</v>
-      </c>
-      <c r="F18" t="s">
-        <v>68</v>
-      </c>
-      <c r="G18" t="s">
-        <v>64</v>
-      </c>
       <c r="H18" t="s">
         <v>18</v>
       </c>
       <c r="I18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
         <v>70</v>
       </c>
-      <c r="C19" t="s">
-        <v>66</v>
-      </c>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G19" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="H19" t="s">
         <v>18</v>
       </c>
       <c r="I19" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E20" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F20" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G20" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="H20" t="s">
         <v>18</v>
       </c>
       <c r="I20" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E21" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="G21" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="H21" t="s">
         <v>18</v>
       </c>
       <c r="I21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" t="s">
         <v>21</v>
       </c>
-      <c r="C22" t="s">
-        <v>24</v>
-      </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="F22" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="G22" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="H22" t="s">
         <v>18</v>
       </c>
       <c r="I22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="15">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="D23" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" t="s">
         <v>72</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>73</v>
       </c>
-      <c r="F23" t="s">
-        <v>74</v>
-      </c>
       <c r="G23" t="s">
-        <v>75</v>
+        <v>29</v>
       </c>
       <c r="H23" t="s">
         <v>18</v>
       </c>
       <c r="I23" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="15">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="D24" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F24" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="G24" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="H24" t="s">
         <v>18</v>
       </c>
       <c r="I24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="15">
       <c r="A25" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="D25" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E25" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F25" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="G25" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="H25" t="s">
         <v>18</v>
       </c>
       <c r="I25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="15">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D26" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="E26" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="F26" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="G26" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="H26" t="s">
         <v>18</v>
       </c>
       <c r="I26" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="15">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="D27" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="E27" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="F27" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="G27" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="H27" t="s">
         <v>18</v>
       </c>
       <c r="I27" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="15">
       <c r="A28" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="D28" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="E28" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="F28" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="G28" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="H28" t="s">
         <v>18</v>
       </c>
       <c r="I28" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="15">
       <c r="A29" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="D29" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E29" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="F29" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="G29" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="H29" t="s">
         <v>18</v>
       </c>
       <c r="I29" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="15">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B30" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="D30" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E30" t="s">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="F30" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="G30" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H30" t="s">
         <v>18</v>
       </c>
       <c r="I30" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="15">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B31" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="D31" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="E31" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="F31" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="G31" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="H31" t="s">
         <v>18</v>
       </c>
       <c r="I31" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="15">
       <c r="A32" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C32" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="E32" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="F32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G32" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="H32" t="s">
         <v>18</v>
       </c>
       <c r="I32" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="15">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B33" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C33" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="D33" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="E33" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="F33" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="G33" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="H33" t="s">
         <v>18</v>
       </c>
       <c r="I33" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="15">
       <c r="A34" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B34" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="D34" t="s">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E34" t="s">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="F34" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="G34" t="s">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="H34" t="s">
         <v>18</v>
       </c>
       <c r="I34" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="15">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B35" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="C35" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="D35" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="E35" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="F35" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="G35" t="s">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="H35" t="s">
         <v>18</v>
       </c>
       <c r="I35" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="15">
       <c r="A36" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C36" t="s">
-        <v>32</v>
+        <v>67</v>
       </c>
       <c r="D36" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E36" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="F36" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="G36" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="H36" t="s">
         <v>18</v>
       </c>
       <c r="I36" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="15">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B37" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C37" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D37" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E37" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F37" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G37" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H37" t="s">
         <v>18</v>
       </c>
       <c r="I37" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C38" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="D38" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="E38" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F38" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="G38" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H38" t="s">
         <v>18</v>
       </c>
       <c r="I38" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="15">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B39" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C39" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="D39" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E39" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F39" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="G39" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="H39" t="s">
         <v>18</v>
       </c>
       <c r="I39" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="15">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B40" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="C40" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="D40" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E40" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F40" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G40" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H40" t="s">
         <v>18</v>
       </c>
       <c r="I40" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="15">
       <c r="A41" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="D41" t="s">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="E41" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="F41" t="s">
-        <v>97</v>
+        <v>42</v>
       </c>
       <c r="G41" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="H41" t="s">
         <v>18</v>
       </c>
       <c r="I41" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="15">
       <c r="A42" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="B42" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="C42" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="D42" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="E42" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="F42" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="G42" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="H42" t="s">
         <v>18</v>
       </c>
       <c r="I42" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="15">
       <c r="A43" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="B43" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="C43" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="D43" t="s">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="E43" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F43" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="G43" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="H43" t="s">
         <v>18</v>
       </c>
       <c r="I43" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="15">
       <c r="A44" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B44" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C44" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D44" t="s">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="E44" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="F44" t="s">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="G44" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="H44" t="s">
         <v>18</v>
       </c>
       <c r="I44" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="15">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B45" t="s">
         <v>20</v>
       </c>
       <c r="C45" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D45" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="E45" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F45" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="G45" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H45" t="s">
         <v>18</v>
       </c>
       <c r="I45" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="15">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B46" t="s">
+        <v>26</v>
+      </c>
+      <c r="C46" t="s">
         <v>21</v>
       </c>
-      <c r="C46" t="s">
-        <v>81</v>
-      </c>
       <c r="D46" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="E46" t="s">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="F46" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="G46" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H46" t="s">
         <v>18</v>
       </c>
       <c r="I46" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="15">
       <c r="A47" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B47" t="s">
+        <v>32</v>
+      </c>
+      <c r="C47" t="s">
         <v>21</v>
       </c>
-      <c r="C47" t="s">
-        <v>24</v>
-      </c>
       <c r="D47" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E47" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="F47" t="s">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="G47" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="H47" t="s">
         <v>18</v>
       </c>
       <c r="I47" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="15">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B48" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="C48" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="D48" t="s">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="E48" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="F48" t="s">
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="G48" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="H48" t="s">
         <v>18</v>
       </c>
       <c r="I48" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="15">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B49" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="C49" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="D49" t="s">
-        <v>105</v>
+        <v>57</v>
       </c>
       <c r="E49" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="F49" t="s">
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="G49" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="H49" t="s">
         <v>18</v>
       </c>
       <c r="I49" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="15">
       <c r="A50" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B50" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="D50" t="s">
-        <v>106</v>
+        <v>57</v>
       </c>
       <c r="E50" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="F50" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="G50" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="H50" t="s">
         <v>18</v>
       </c>
       <c r="I50" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="15">
       <c r="A51" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B51" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C51" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>107</v>
+        <v>14</v>
       </c>
       <c r="E51" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F51" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="G51" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="H51" t="s">
         <v>18</v>
       </c>
       <c r="I51" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="15">
       <c r="A52" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B52" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C52" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D52" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="E52" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="F52" t="s">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="G52" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="H52" t="s">
         <v>18</v>
       </c>
       <c r="I52" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="15">
       <c r="A53" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B53" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C53" t="s">
         <v>13</v>
@@ -2519,1208 +2404,744 @@
         <v>14</v>
       </c>
       <c r="E53" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="F53" t="s">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="G53" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H53" t="s">
         <v>18</v>
       </c>
       <c r="I53" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="15">
       <c r="A54" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B54" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C54" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="D54" t="s">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="E54" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="F54" t="s">
-        <v>110</v>
+        <v>28</v>
       </c>
       <c r="G54" t="s">
-        <v>111</v>
+        <v>30</v>
       </c>
       <c r="H54" t="s">
         <v>18</v>
       </c>
       <c r="I54" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="15">
       <c r="A55" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B55" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C55" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D55" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E55" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F55" t="s">
-        <v>97</v>
+        <v>16</v>
       </c>
       <c r="G55" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="H55" t="s">
         <v>18</v>
       </c>
       <c r="I55" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="15">
       <c r="A56" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B56" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C56" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D56" t="s">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="E56" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F56" t="s">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="G56" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H56" t="s">
         <v>18</v>
       </c>
       <c r="I56" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="15">
       <c r="A57" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B57" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C57" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
       <c r="D57" t="s">
-        <v>113</v>
+        <v>14</v>
       </c>
       <c r="E57" t="s">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="F57" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="G57" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
       <c r="H57" t="s">
         <v>18</v>
       </c>
       <c r="I57" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="15">
       <c r="A58" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B58" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="D58" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="E58" t="s">
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="F58" t="s">
-        <v>92</v>
+        <v>16</v>
       </c>
       <c r="G58" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="H58" t="s">
         <v>18</v>
       </c>
       <c r="I58" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="15">
       <c r="A59" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B59" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C59" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D59" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E59" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F59" t="s">
-        <v>97</v>
+        <v>16</v>
       </c>
       <c r="G59" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="H59" t="s">
         <v>18</v>
       </c>
       <c r="I59" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="15">
       <c r="A60" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B60" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C60" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="D60" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="E60" t="s">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="F60" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="G60" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H60" t="s">
         <v>18</v>
       </c>
       <c r="I60" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="15">
       <c r="A61" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B61" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C61" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D61" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E61" t="s">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="F61" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G61" t="s">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="H61" t="s">
         <v>18</v>
       </c>
       <c r="I61" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="62" spans="1:9" ht="15">
       <c r="A62" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B62" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C62" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="D62" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="E62" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="F62" t="s">
-        <v>110</v>
+        <v>54</v>
       </c>
       <c r="G62" t="s">
-        <v>116</v>
+        <v>30</v>
       </c>
       <c r="H62" t="s">
         <v>18</v>
       </c>
       <c r="I62" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="15">
       <c r="A63" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B63" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="C63" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="D63" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E63" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="F63" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="G63" t="s">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="H63" t="s">
         <v>18</v>
       </c>
       <c r="I63" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="15">
       <c r="A64" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B64" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="C64" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="D64" t="s">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="E64" t="s">
-        <v>117</v>
+        <v>27</v>
       </c>
       <c r="F64" t="s">
-        <v>110</v>
+        <v>28</v>
       </c>
       <c r="G64" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="H64" t="s">
         <v>18</v>
       </c>
       <c r="I64" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="15">
       <c r="A65" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B65" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="C65" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D65" t="s">
-        <v>115</v>
+        <v>44</v>
       </c>
       <c r="E65" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F65" t="s">
-        <v>97</v>
+        <v>16</v>
       </c>
       <c r="G65" t="s">
-        <v>116</v>
+        <v>30</v>
       </c>
       <c r="H65" t="s">
         <v>18</v>
       </c>
       <c r="I65" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="15">
       <c r="A66" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B66" t="s">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="C66" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="E66" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="F66" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="G66" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="H66" t="s">
         <v>18</v>
       </c>
       <c r="I66" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="15">
       <c r="A67" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B67" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="D67" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E67" t="s">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="F67" t="s">
-        <v>110</v>
+        <v>28</v>
       </c>
       <c r="G67" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="H67" t="s">
         <v>18</v>
       </c>
       <c r="I67" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="15">
       <c r="A68" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B68" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="C68" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D68" t="s">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="E68" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="F68" t="s">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="G68" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H68" t="s">
         <v>18</v>
       </c>
       <c r="I68" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="15">
       <c r="A69" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B69" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="C69" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="D69" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="E69" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="F69" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="G69" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="H69" t="s">
         <v>18</v>
       </c>
       <c r="I69" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="15">
       <c r="A70" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B70" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="C70" t="s">
-        <v>118</v>
+        <v>21</v>
       </c>
       <c r="D70" t="s">
-        <v>121</v>
+        <v>40</v>
       </c>
       <c r="E70" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="F70" t="s">
-        <v>120</v>
+        <v>28</v>
       </c>
       <c r="G70" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="H70" t="s">
         <v>18</v>
       </c>
       <c r="I70" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="15">
       <c r="A71" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B71" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="C71" t="s">
         <v>13</v>
       </c>
       <c r="D71" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E71" t="s">
-        <v>123</v>
+        <v>38</v>
       </c>
       <c r="F71" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="G71" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H71" t="s">
         <v>18</v>
       </c>
       <c r="I71" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="15">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B72" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C72" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="D72" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E72" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="F72" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="G72" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="H72" t="s">
         <v>18</v>
       </c>
       <c r="I72" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="15">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B73" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C73" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="D73" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="E73" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F73" t="s">
-        <v>125</v>
+        <v>28</v>
       </c>
       <c r="G73" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="H73" t="s">
         <v>18</v>
       </c>
       <c r="I73" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="15">
       <c r="A74" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B74" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C74" t="s">
         <v>13</v>
       </c>
       <c r="D74" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E74" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="F74" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="G74" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H74" t="s">
         <v>18</v>
       </c>
       <c r="I74" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="15">
       <c r="A75" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B75" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="D75" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="E75" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="F75" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="G75" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="H75" t="s">
         <v>18</v>
       </c>
       <c r="I75" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="15">
       <c r="A76" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B76" t="s">
+        <v>45</v>
+      </c>
+      <c r="C76" t="s">
         <v>21</v>
       </c>
-      <c r="C76" t="s">
-        <v>81</v>
-      </c>
       <c r="D76" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E76" t="s">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="F76" t="s">
-        <v>110</v>
+        <v>28</v>
       </c>
       <c r="G76" t="s">
-        <v>126</v>
+        <v>30</v>
       </c>
       <c r="H76" t="s">
         <v>18</v>
       </c>
       <c r="I76" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="15">
       <c r="A77" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B77" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C77" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D77" t="s">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="E77" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F77" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G77" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H77" t="s">
         <v>18</v>
       </c>
       <c r="I77" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="15">
       <c r="A78" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B78" t="s">
+        <v>47</v>
+      </c>
+      <c r="C78" t="s">
         <v>21</v>
       </c>
-      <c r="C78" t="s">
-        <v>13</v>
-      </c>
       <c r="D78" t="s">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="E78" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F78" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="G78" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="H78" t="s">
         <v>18</v>
       </c>
       <c r="I78" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" ht="15">
-      <c r="A79" t="s">
-        <v>122</v>
-      </c>
-      <c r="B79" t="s">
-        <v>23</v>
-      </c>
-      <c r="C79" t="s">
-        <v>81</v>
-      </c>
-      <c r="D79" t="s">
-        <v>46</v>
-      </c>
-      <c r="E79" t="s">
-        <v>36</v>
-      </c>
-      <c r="F79" t="s">
-        <v>37</v>
-      </c>
-      <c r="G79" t="s">
-        <v>60</v>
-      </c>
-      <c r="H79" t="s">
-        <v>18</v>
-      </c>
-      <c r="I79" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" ht="15">
-      <c r="A80" t="s">
-        <v>122</v>
-      </c>
-      <c r="B80" t="s">
-        <v>23</v>
-      </c>
-      <c r="C80" t="s">
-        <v>24</v>
-      </c>
-      <c r="D80" t="s">
-        <v>96</v>
-      </c>
-      <c r="E80" t="s">
-        <v>47</v>
-      </c>
-      <c r="F80" t="s">
-        <v>125</v>
-      </c>
-      <c r="G80" t="s">
-        <v>98</v>
-      </c>
-      <c r="H80" t="s">
-        <v>18</v>
-      </c>
-      <c r="I80" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" ht="15">
-      <c r="A81" t="s">
-        <v>122</v>
-      </c>
-      <c r="B81" t="s">
-        <v>23</v>
-      </c>
-      <c r="C81" t="s">
-        <v>13</v>
-      </c>
-      <c r="D81" t="s">
-        <v>40</v>
-      </c>
-      <c r="E81" t="s">
-        <v>30</v>
-      </c>
-      <c r="F81" t="s">
-        <v>68</v>
-      </c>
-      <c r="G81" t="s">
-        <v>99</v>
-      </c>
-      <c r="H81" t="s">
-        <v>18</v>
-      </c>
-      <c r="I81" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" ht="15">
-      <c r="A82" t="s">
-        <v>122</v>
-      </c>
-      <c r="B82" t="s">
-        <v>31</v>
-      </c>
-      <c r="C82" t="s">
-        <v>124</v>
-      </c>
-      <c r="D82" t="s">
-        <v>127</v>
-      </c>
-      <c r="E82" t="s">
-        <v>117</v>
-      </c>
-      <c r="F82" t="s">
-        <v>112</v>
-      </c>
-      <c r="G82" t="s">
-        <v>17</v>
-      </c>
-      <c r="H82" t="s">
-        <v>18</v>
-      </c>
-      <c r="I82" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" ht="15">
-      <c r="A83" t="s">
-        <v>122</v>
-      </c>
-      <c r="B83" t="s">
-        <v>31</v>
-      </c>
-      <c r="C83" t="s">
-        <v>81</v>
-      </c>
-      <c r="D83" t="s">
-        <v>128</v>
-      </c>
-      <c r="E83" t="s">
-        <v>89</v>
-      </c>
-      <c r="F83" t="s">
-        <v>68</v>
-      </c>
-      <c r="G83" t="s">
-        <v>129</v>
-      </c>
-      <c r="H83" t="s">
-        <v>18</v>
-      </c>
-      <c r="I83" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" ht="15">
-      <c r="A84" t="s">
-        <v>122</v>
-      </c>
-      <c r="B84" t="s">
-        <v>31</v>
-      </c>
-      <c r="C84" t="s">
-        <v>24</v>
-      </c>
-      <c r="D84" t="s">
-        <v>91</v>
-      </c>
-      <c r="E84" t="s">
-        <v>47</v>
-      </c>
-      <c r="F84" t="s">
-        <v>48</v>
-      </c>
-      <c r="G84" t="s">
-        <v>17</v>
-      </c>
-      <c r="H84" t="s">
-        <v>18</v>
-      </c>
-      <c r="I84" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" ht="15">
-      <c r="A85" t="s">
-        <v>122</v>
-      </c>
-      <c r="B85" t="s">
-        <v>31</v>
-      </c>
-      <c r="C85" t="s">
-        <v>13</v>
-      </c>
-      <c r="D85" t="s">
-        <v>40</v>
-      </c>
-      <c r="E85" t="s">
-        <v>30</v>
-      </c>
-      <c r="F85" t="s">
-        <v>112</v>
-      </c>
-      <c r="G85" t="s">
-        <v>99</v>
-      </c>
-      <c r="H85" t="s">
-        <v>18</v>
-      </c>
-      <c r="I85" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" ht="15">
-      <c r="A86" t="s">
-        <v>122</v>
-      </c>
-      <c r="B86" t="s">
-        <v>44</v>
-      </c>
-      <c r="C86" t="s">
-        <v>124</v>
-      </c>
-      <c r="D86" t="s">
-        <v>130</v>
-      </c>
-      <c r="E86" t="s">
-        <v>36</v>
-      </c>
-      <c r="F86" t="s">
-        <v>37</v>
-      </c>
-      <c r="G86" t="s">
-        <v>38</v>
-      </c>
-      <c r="H86" t="s">
-        <v>18</v>
-      </c>
-      <c r="I86" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" ht="15">
-      <c r="A87" t="s">
-        <v>122</v>
-      </c>
-      <c r="B87" t="s">
-        <v>44</v>
-      </c>
-      <c r="C87" t="s">
-        <v>81</v>
-      </c>
-      <c r="D87" t="s">
-        <v>85</v>
-      </c>
-      <c r="E87" t="s">
-        <v>89</v>
-      </c>
-      <c r="F87" t="s">
-        <v>68</v>
-      </c>
-      <c r="G87" t="s">
-        <v>126</v>
-      </c>
-      <c r="H87" t="s">
-        <v>18</v>
-      </c>
-      <c r="I87" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" ht="15">
-      <c r="A88" t="s">
-        <v>122</v>
-      </c>
-      <c r="B88" t="s">
-        <v>44</v>
-      </c>
-      <c r="C88" t="s">
-        <v>24</v>
-      </c>
-      <c r="D88" t="s">
-        <v>91</v>
-      </c>
-      <c r="E88" t="s">
-        <v>47</v>
-      </c>
-      <c r="F88" t="s">
-        <v>48</v>
-      </c>
-      <c r="G88" t="s">
-        <v>17</v>
-      </c>
-      <c r="H88" t="s">
-        <v>18</v>
-      </c>
-      <c r="I88" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" ht="15">
-      <c r="A89" t="s">
-        <v>122</v>
-      </c>
-      <c r="B89" t="s">
-        <v>44</v>
-      </c>
-      <c r="C89" t="s">
-        <v>13</v>
-      </c>
-      <c r="D89" t="s">
-        <v>40</v>
-      </c>
-      <c r="E89" t="s">
-        <v>50</v>
-      </c>
-      <c r="F89" t="s">
-        <v>112</v>
-      </c>
-      <c r="G89" t="s">
-        <v>99</v>
-      </c>
-      <c r="H89" t="s">
-        <v>18</v>
-      </c>
-      <c r="I89" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" ht="15">
-      <c r="A90" t="s">
-        <v>122</v>
-      </c>
-      <c r="B90" t="s">
-        <v>53</v>
-      </c>
-      <c r="C90" t="s">
-        <v>124</v>
-      </c>
-      <c r="D90" t="s">
-        <v>131</v>
-      </c>
-      <c r="E90" t="s">
-        <v>36</v>
-      </c>
-      <c r="F90" t="s">
-        <v>37</v>
-      </c>
-      <c r="G90" t="s">
-        <v>38</v>
-      </c>
-      <c r="H90" t="s">
-        <v>18</v>
-      </c>
-      <c r="I90" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" ht="15">
-      <c r="A91" t="s">
-        <v>122</v>
-      </c>
-      <c r="B91" t="s">
-        <v>53</v>
-      </c>
-      <c r="C91" t="s">
-        <v>81</v>
-      </c>
-      <c r="D91" t="s">
-        <v>113</v>
-      </c>
-      <c r="E91" t="s">
-        <v>89</v>
-      </c>
-      <c r="F91" t="s">
-        <v>68</v>
-      </c>
-      <c r="G91" t="s">
-        <v>129</v>
-      </c>
-      <c r="H91" t="s">
-        <v>18</v>
-      </c>
-      <c r="I91" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" ht="15">
-      <c r="A92" t="s">
-        <v>122</v>
-      </c>
-      <c r="B92" t="s">
-        <v>53</v>
-      </c>
-      <c r="C92" t="s">
-        <v>24</v>
-      </c>
-      <c r="D92" t="s">
-        <v>115</v>
-      </c>
-      <c r="E92" t="s">
-        <v>50</v>
-      </c>
-      <c r="F92" t="s">
-        <v>132</v>
-      </c>
-      <c r="G92" t="s">
-        <v>35</v>
-      </c>
-      <c r="H92" t="s">
-        <v>18</v>
-      </c>
-      <c r="I92" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9" ht="15">
-      <c r="A93" t="s">
-        <v>122</v>
-      </c>
-      <c r="B93" t="s">
-        <v>54</v>
-      </c>
-      <c r="C93" t="s">
-        <v>24</v>
-      </c>
-      <c r="D93" t="s">
-        <v>115</v>
-      </c>
-      <c r="E93" t="s">
-        <v>133</v>
-      </c>
-      <c r="F93" t="s">
-        <v>134</v>
-      </c>
-      <c r="G93" t="s">
-        <v>135</v>
-      </c>
-      <c r="H93" t="s">
-        <v>18</v>
-      </c>
-      <c r="I93" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="94" spans="1:9" ht="15">
-      <c r="A94" t="s">
-        <v>122</v>
-      </c>
-      <c r="B94" t="s">
-        <v>61</v>
-      </c>
-      <c r="C94" t="s">
-        <v>24</v>
-      </c>
-      <c r="D94" t="s">
-        <v>115</v>
-      </c>
-      <c r="E94" t="s">
-        <v>133</v>
-      </c>
-      <c r="F94" t="s">
-        <v>134</v>
-      </c>
-      <c r="G94" t="s">
-        <v>135</v>
-      </c>
-      <c r="H94" t="s">
-        <v>18</v>
-      </c>
-      <c r="I94" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -3731,13 +3152,152 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{5f4407a8-5b32-4469-94ef-9f5ffad6c2ad}">
-  <dimension ref="A1:F19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{c43d19c3-00f8-43fd-bbf0-6a5019495413}">
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
     <col min="2" max="2" width="11.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="17.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="18.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="36.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="15.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="7.42857142857143" customWidth="1"/>
+    <col min="7" max="7" width="45.5714285714286" customWidth="1"/>
+    <col min="8" max="8" width="9.28571428571429" customWidth="1"/>
+    <col min="9" max="9" width="17.8571428571429" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="56.25" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="15">
+      <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{a7d12d72-5462-41e7-838e-42a1c7885cf9}">
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
+    <col min="2" max="2" width="11.1428571428571" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="35.1428571428571" customWidth="1"/>
     <col min="5" max="5" width="28.1428571428571" customWidth="1"/>
     <col min="6" max="6" width="9.28571428571429" customWidth="1"/>
@@ -3748,13 +3308,13 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>136</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>137</v>
+        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>138</v>
+        <v>107</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -3768,16 +3328,16 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>108</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>140</v>
+        <v>109</v>
       </c>
       <c r="E2" t="s">
-        <v>141</v>
+        <v>110</v>
       </c>
       <c r="F2" t="s">
         <v>18</v>
@@ -3788,16 +3348,16 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="E3" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -3808,16 +3368,16 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>140</v>
+        <v>114</v>
       </c>
       <c r="E4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
@@ -3825,19 +3385,19 @@
     </row>
     <row r="5" spans="1:6" ht="15">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>116</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>145</v>
+        <v>117</v>
       </c>
       <c r="E5" t="s">
-        <v>146</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
         <v>18</v>
@@ -3845,19 +3405,19 @@
     </row>
     <row r="6" spans="1:6" ht="15">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="D6" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
         <v>18</v>
@@ -3865,19 +3425,19 @@
     </row>
     <row r="7" spans="1:6" ht="15">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>149</v>
+        <v>113</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>117</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
         <v>18</v>
@@ -3885,19 +3445,19 @@
     </row>
     <row r="8" spans="1:6" ht="15">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="B8" t="s">
-        <v>151</v>
+        <v>118</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>152</v>
+        <v>109</v>
       </c>
       <c r="E8" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
         <v>18</v>
@@ -3905,19 +3465,19 @@
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="B9" t="s">
-        <v>153</v>
+        <v>119</v>
       </c>
       <c r="C9" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="E9" t="s">
-        <v>154</v>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
         <v>18</v>
@@ -3925,19 +3485,19 @@
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>153</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
       <c r="E10" t="s">
-        <v>116</v>
+        <v>30</v>
       </c>
       <c r="F10" t="s">
         <v>18</v>
@@ -3945,19 +3505,19 @@
     </row>
     <row r="11" spans="1:6" ht="15">
       <c r="A11" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="B11" t="s">
-        <v>155</v>
+        <v>122</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="E11" t="s">
-        <v>156</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
         <v>18</v>
@@ -3965,19 +3525,19 @@
     </row>
     <row r="12" spans="1:6" ht="15">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>111</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>157</v>
+        <v>109</v>
       </c>
       <c r="E12" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F12" t="s">
         <v>18</v>
@@ -3985,19 +3545,19 @@
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="C13" t="s">
-        <v>124</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>157</v>
+        <v>109</v>
       </c>
       <c r="E13" t="s">
-        <v>158</v>
+        <v>30</v>
       </c>
       <c r="F13" t="s">
         <v>18</v>
@@ -4005,19 +3565,19 @@
     </row>
     <row r="14" spans="1:6" ht="15">
       <c r="A14" t="s">
-        <v>122</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="C14" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>157</v>
+        <v>114</v>
       </c>
       <c r="E14" t="s">
-        <v>159</v>
+        <v>30</v>
       </c>
       <c r="F14" t="s">
         <v>18</v>
@@ -4025,19 +3585,19 @@
     </row>
     <row r="15" spans="1:6" ht="15">
       <c r="A15" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B15" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D15" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="E15" t="s">
-        <v>160</v>
+        <v>30</v>
       </c>
       <c r="F15" t="s">
         <v>18</v>
@@ -4045,19 +3605,19 @@
     </row>
     <row r="16" spans="1:6" ht="15">
       <c r="A16" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B16" t="s">
-        <v>155</v>
+        <v>123</v>
       </c>
       <c r="C16" t="s">
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>140</v>
+        <v>114</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
@@ -4065,19 +3625,19 @@
     </row>
     <row r="17" spans="1:6" ht="15">
       <c r="A17" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B17" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="D17" t="s">
-        <v>150</v>
+        <v>114</v>
       </c>
       <c r="E17" t="s">
-        <v>161</v>
+        <v>30</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -4085,41 +3645,21 @@
     </row>
     <row r="18" spans="1:6" ht="15">
       <c r="A18" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B18" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="C18" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D18" t="s">
-        <v>152</v>
+        <v>109</v>
       </c>
       <c r="E18" t="s">
-        <v>162</v>
+        <v>30</v>
       </c>
       <c r="F18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15">
-      <c r="A19" t="s">
-        <v>122</v>
-      </c>
-      <c r="B19" t="s">
-        <v>163</v>
-      </c>
-      <c r="C19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" t="s">
-        <v>152</v>
-      </c>
-      <c r="E19" t="s">
-        <v>116</v>
-      </c>
-      <c r="F19" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cover Katarzyna Świerzewicz's Friday absence
Refreshed substitutions for the same 14-30.09.2026 package: 182 entries,
31 duty replacements and 8 other-activity entries. Everything outside
18.09 is unchanged.

On 18.09 the four "Okienko dla uczniów" gaps in 2K become substituted
lessons and three more lessons are covered, 2K lesson 1 and 1K lessons 6
and 7. A special-educator duty and one corridor duty are added.

Eight diary names were removed with scripts/privacy_xlsx.py before the
commit; no other cell differs from the source export.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSteHAUcpUZjXBcPeyJY4A
</commit_message>
<xml_diff>
--- a/InformacjeOZastepstwach.xlsx
+++ b/InformacjeOZastepstwach.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<s:sst xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="225">
+<s:sst xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="232">
   <s:si>
     <s:t>Rok szkolny: 2026/2027</s:t>
   </s:si>
@@ -432,6 +432,15 @@
     <s:t>18.09.2026</s:t>
   </s:si>
   <s:si>
+    <s:t>Świerzewicz Katarzyna</s:t>
+  </s:si>
+  <s:si>
+    <s:t>2K</s:t>
+  </s:si>
+  <s:si>
+    <s:t>Technologia gastronomiczna z towaroznawstwem</s:t>
+  </s:si>
+  <s:si>
     <s:t>1FB|gr2</s:t>
   </s:si>
   <s:si>
@@ -441,15 +450,6 @@
     <s:t>Jastrzębska-Majtyka Agnieszka</s:t>
   </s:si>
   <s:si>
-    <s:t>Świerzewicz Katarzyna</s:t>
-  </s:si>
-  <s:si>
-    <s:t>2K</s:t>
-  </s:si>
-  <s:si>
-    <s:t>Technologia gastronomiczna z towaroznawstwem</s:t>
-  </s:si>
-  <s:si>
     <s:t>1TFH|gr2</s:t>
   </s:si>
   <s:si>
@@ -486,6 +486,12 @@
     <s:t>Informatyka</s:t>
   </s:si>
   <s:si>
+    <s:t>1K</s:t>
+  </s:si>
+  <s:si>
+    <s:t>Mocarski Arkadiusz</s:t>
+  </s:si>
+  <s:si>
     <s:t>41</s:t>
   </s:si>
   <s:si>
@@ -498,6 +504,9 @@
     <s:t>27</s:t>
   </s:si>
   <s:si>
+    <s:t>Rozwój kompetencji zawodowych - Zasady zdrowego żywienia</s:t>
+  </s:si>
+  <s:si>
     <s:t>4</s:t>
   </s:si>
   <s:si>
@@ -552,9 +561,6 @@
     <s:t>Biznes i zarządzanie</s:t>
   </s:si>
   <s:si>
-    <s:t>1K</s:t>
-  </s:si>
-  <s:si>
     <s:t>1WB</s:t>
   </s:si>
   <s:si>
@@ -630,6 +636,18 @@
     <s:t>Dyżur psychologa szkolnego</s:t>
   </s:si>
   <s:si>
+    <s:t>09:00-13:00</s:t>
+  </s:si>
+  <s:si>
+    <s:t>Kaszak Maria</s:t>
+  </s:si>
+  <s:si>
+    <s:t/>
+  </s:si>
+  <s:si>
+    <s:t xml:space="preserve">dyżur pedagoga specjalnego </s:t>
+  </s:si>
+  <s:si>
     <s:t xml:space="preserve">Matematyka </s:t>
   </s:si>
   <s:si>
@@ -667,6 +685,9 @@
   </s:si>
   <s:si>
     <s:t>13:10-13:15</s:t>
+  </s:si>
+  <s:si>
+    <s:t>07:55-08:00</s:t>
   </s:si>
   <s:si>
     <s:t>08:45-08:50</s:t>
@@ -1146,7 +1167,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{fa50b800-9567-4135-a9f7-c76c650b0a31}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{7acacd02-a3f5-4dae-9df1-d08e1d54cfba}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -1167,8 +1188,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{1c5b9002-c574-42cb-8730-6575dba92b7b}">
-  <dimension ref="A1:I180"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{05501696-feab-4fce-affd-2617c323f72e}">
+  <dimension ref="A1:I183"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
@@ -3536,19 +3557,19 @@
         <v>135</v>
       </c>
       <c r="B82" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C82" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D82" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E82" t="s">
-        <v>92</v>
+        <v>138</v>
       </c>
       <c r="F82" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="G82" t="s">
         <v>113</v>
@@ -3568,25 +3589,25 @@
         <v>20</v>
       </c>
       <c r="C83" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D83" t="s">
-        <v>51</v>
+        <v>139</v>
       </c>
       <c r="E83" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="F83" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="G83" t="s">
-        <v>138</v>
+        <v>113</v>
       </c>
       <c r="H83" t="s">
         <v>18</v>
       </c>
       <c r="I83" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="84" spans="1:9" ht="15">
@@ -3597,19 +3618,19 @@
         <v>20</v>
       </c>
       <c r="C84" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D84" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="E84" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="F84" t="s">
-        <v>16</v>
+        <v>121</v>
       </c>
       <c r="G84" t="s">
-        <v>17</v>
+        <v>141</v>
       </c>
       <c r="H84" t="s">
         <v>18</v>
@@ -3626,25 +3647,25 @@
         <v>20</v>
       </c>
       <c r="C85" t="s">
-        <v>139</v>
+        <v>13</v>
       </c>
       <c r="D85" t="s">
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="E85" t="s">
-        <v>141</v>
+        <v>37</v>
       </c>
       <c r="F85" t="s">
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="G85" t="s">
-        <v>133</v>
+        <v>17</v>
       </c>
       <c r="H85" t="s">
         <v>18</v>
       </c>
       <c r="I85" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="86" spans="1:9" ht="15">
@@ -3652,28 +3673,28 @@
         <v>135</v>
       </c>
       <c r="B86" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C86" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D86" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E86" t="s">
-        <v>69</v>
+        <v>138</v>
       </c>
       <c r="F86" t="s">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="G86" t="s">
-        <v>127</v>
+        <v>28</v>
       </c>
       <c r="H86" t="s">
         <v>18</v>
       </c>
       <c r="I86" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="87" spans="1:9" ht="15">
@@ -3684,19 +3705,19 @@
         <v>26</v>
       </c>
       <c r="C87" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D87" t="s">
-        <v>116</v>
+        <v>142</v>
       </c>
       <c r="E87" t="s">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="F87" t="s">
-        <v>143</v>
+        <v>53</v>
       </c>
       <c r="G87" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="H87" t="s">
         <v>18</v>
@@ -3713,19 +3734,19 @@
         <v>26</v>
       </c>
       <c r="C88" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D88" t="s">
-        <v>43</v>
+        <v>116</v>
       </c>
       <c r="E88" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="F88" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="G88" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="H88" t="s">
         <v>18</v>
@@ -3742,25 +3763,25 @@
         <v>26</v>
       </c>
       <c r="C89" t="s">
-        <v>139</v>
+        <v>13</v>
       </c>
       <c r="D89" t="s">
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="E89" t="s">
-        <v>141</v>
+        <v>37</v>
       </c>
       <c r="F89" t="s">
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="G89" t="s">
-        <v>133</v>
+        <v>17</v>
       </c>
       <c r="H89" t="s">
         <v>18</v>
       </c>
       <c r="I89" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="90" spans="1:9" ht="15">
@@ -3768,28 +3789,28 @@
         <v>135</v>
       </c>
       <c r="B90" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C90" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D90" t="s">
-        <v>51</v>
+        <v>137</v>
       </c>
       <c r="E90" t="s">
-        <v>47</v>
+        <v>138</v>
       </c>
       <c r="F90" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="G90" t="s">
-        <v>146</v>
+        <v>28</v>
       </c>
       <c r="H90" t="s">
         <v>18</v>
       </c>
       <c r="I90" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="91" spans="1:9" ht="15">
@@ -3800,19 +3821,19 @@
         <v>31</v>
       </c>
       <c r="C91" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D91" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="E91" t="s">
-        <v>147</v>
+        <v>47</v>
       </c>
       <c r="F91" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G91" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H91" t="s">
         <v>18</v>
@@ -3829,19 +3850,19 @@
         <v>31</v>
       </c>
       <c r="C92" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="D92" t="s">
-        <v>150</v>
+        <v>39</v>
       </c>
       <c r="E92" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F92" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="G92" t="s">
-        <v>94</v>
+        <v>149</v>
       </c>
       <c r="H92" t="s">
         <v>18</v>
@@ -3858,25 +3879,25 @@
         <v>31</v>
       </c>
       <c r="C93" t="s">
-        <v>144</v>
+        <v>59</v>
       </c>
       <c r="D93" t="s">
-        <v>56</v>
+        <v>150</v>
       </c>
       <c r="E93" t="s">
-        <v>23</v>
+        <v>151</v>
       </c>
       <c r="F93" t="s">
-        <v>143</v>
+        <v>109</v>
       </c>
       <c r="G93" t="s">
-        <v>28</v>
+        <v>94</v>
       </c>
       <c r="H93" t="s">
         <v>18</v>
       </c>
       <c r="I93" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="94" spans="1:9" ht="15">
@@ -3887,25 +3908,25 @@
         <v>31</v>
       </c>
       <c r="C94" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="D94" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="E94" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="F94" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="G94" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H94" t="s">
         <v>18</v>
       </c>
       <c r="I94" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="95" spans="1:9" ht="15">
@@ -3916,25 +3937,25 @@
         <v>31</v>
       </c>
       <c r="C95" t="s">
-        <v>139</v>
+        <v>13</v>
       </c>
       <c r="D95" t="s">
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="E95" t="s">
-        <v>141</v>
+        <v>37</v>
       </c>
       <c r="F95" t="s">
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="G95" t="s">
-        <v>133</v>
+        <v>17</v>
       </c>
       <c r="H95" t="s">
         <v>18</v>
       </c>
       <c r="I95" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="96" spans="1:9" ht="15">
@@ -3942,28 +3963,28 @@
         <v>135</v>
       </c>
       <c r="B96" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C96" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D96" t="s">
-        <v>51</v>
+        <v>137</v>
       </c>
       <c r="E96" t="s">
-        <v>33</v>
+        <v>138</v>
       </c>
       <c r="F96" t="s">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="G96" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="H96" t="s">
         <v>18</v>
       </c>
       <c r="I96" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="97" spans="1:9" ht="15">
@@ -3974,25 +3995,25 @@
         <v>38</v>
       </c>
       <c r="C97" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D97" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="E97" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="F97" t="s">
-        <v>104</v>
+        <v>34</v>
       </c>
       <c r="G97" t="s">
-        <v>146</v>
+        <v>82</v>
       </c>
       <c r="H97" t="s">
         <v>18</v>
       </c>
       <c r="I97" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="15">
@@ -4003,19 +4024,19 @@
         <v>38</v>
       </c>
       <c r="C98" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="D98" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E98" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="F98" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="G98" t="s">
-        <v>25</v>
+        <v>146</v>
       </c>
       <c r="H98" t="s">
         <v>18</v>
@@ -4032,10 +4053,10 @@
         <v>38</v>
       </c>
       <c r="C99" t="s">
-        <v>144</v>
+        <v>59</v>
       </c>
       <c r="D99" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="E99" t="s">
         <v>23</v>
@@ -4044,13 +4065,13 @@
         <v>143</v>
       </c>
       <c r="G99" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H99" t="s">
         <v>18</v>
       </c>
       <c r="I99" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="100" spans="1:9" ht="15">
@@ -4061,25 +4082,25 @@
         <v>38</v>
       </c>
       <c r="C100" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="D100" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="E100" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="F100" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="G100" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H100" t="s">
         <v>18</v>
       </c>
       <c r="I100" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="101" spans="1:9" ht="15">
@@ -4090,25 +4111,25 @@
         <v>38</v>
       </c>
       <c r="C101" t="s">
-        <v>139</v>
+        <v>13</v>
       </c>
       <c r="D101" t="s">
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="E101" t="s">
-        <v>141</v>
+        <v>37</v>
       </c>
       <c r="F101" t="s">
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="G101" t="s">
-        <v>133</v>
+        <v>17</v>
       </c>
       <c r="H101" t="s">
         <v>18</v>
       </c>
       <c r="I101" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="102" spans="1:9" ht="15">
@@ -4116,28 +4137,28 @@
         <v>135</v>
       </c>
       <c r="B102" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C102" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D102" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="E102" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="F102" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="G102" t="s">
-        <v>146</v>
+        <v>28</v>
       </c>
       <c r="H102" t="s">
         <v>18</v>
       </c>
       <c r="I102" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="103" spans="1:9" ht="15">
@@ -4148,25 +4169,25 @@
         <v>44</v>
       </c>
       <c r="C103" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D103" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="E103" t="s">
-        <v>33</v>
+        <v>153</v>
       </c>
       <c r="F103" t="s">
-        <v>34</v>
+        <v>145</v>
       </c>
       <c r="G103" t="s">
-        <v>82</v>
+        <v>146</v>
       </c>
       <c r="H103" t="s">
         <v>18</v>
       </c>
       <c r="I103" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
     </row>
     <row r="104" spans="1:9" ht="15">
@@ -4177,25 +4198,25 @@
         <v>44</v>
       </c>
       <c r="C104" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="D104" t="s">
-        <v>56</v>
+        <v>114</v>
       </c>
       <c r="E104" t="s">
-        <v>131</v>
+        <v>33</v>
       </c>
       <c r="F104" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="G104" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="H104" t="s">
         <v>18</v>
       </c>
       <c r="I104" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
     </row>
     <row r="105" spans="1:9" ht="15">
@@ -4206,25 +4227,25 @@
         <v>44</v>
       </c>
       <c r="C105" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="D105" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="E105" t="s">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="F105" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="G105" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H105" t="s">
         <v>18</v>
       </c>
       <c r="I105" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="106" spans="1:9" ht="15">
@@ -4232,22 +4253,22 @@
         <v>135</v>
       </c>
       <c r="B106" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C106" t="s">
-        <v>122</v>
+        <v>13</v>
       </c>
       <c r="D106" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="E106" t="s">
-        <v>153</v>
+        <v>47</v>
       </c>
       <c r="F106" t="s">
-        <v>154</v>
+        <v>16</v>
       </c>
       <c r="G106" t="s">
-        <v>146</v>
+        <v>17</v>
       </c>
       <c r="H106" t="s">
         <v>18</v>
@@ -4261,22 +4282,22 @@
         <v>135</v>
       </c>
       <c r="B107" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C107" t="s">
-        <v>21</v>
+        <v>136</v>
       </c>
       <c r="D107" t="s">
+        <v>154</v>
+      </c>
+      <c r="E107" t="s">
+        <v>138</v>
+      </c>
+      <c r="F107" t="s">
+        <v>104</v>
+      </c>
+      <c r="G107" t="s">
         <v>155</v>
-      </c>
-      <c r="E107" t="s">
-        <v>23</v>
-      </c>
-      <c r="F107" t="s">
-        <v>16</v>
-      </c>
-      <c r="G107" t="s">
-        <v>25</v>
       </c>
       <c r="H107" t="s">
         <v>18</v>
@@ -4293,25 +4314,25 @@
         <v>46</v>
       </c>
       <c r="C108" t="s">
-        <v>59</v>
+        <v>122</v>
       </c>
       <c r="D108" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="E108" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="F108" t="s">
-        <v>58</v>
+        <v>156</v>
       </c>
       <c r="G108" t="s">
-        <v>28</v>
+        <v>146</v>
       </c>
       <c r="H108" t="s">
         <v>18</v>
       </c>
       <c r="I108" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="109" spans="1:9" ht="15">
@@ -4322,25 +4343,25 @@
         <v>46</v>
       </c>
       <c r="C109" t="s">
-        <v>144</v>
+        <v>21</v>
       </c>
       <c r="D109" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E109" t="s">
         <v>23</v>
       </c>
       <c r="F109" t="s">
-        <v>157</v>
+        <v>16</v>
       </c>
       <c r="G109" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="H109" t="s">
         <v>18</v>
       </c>
       <c r="I109" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="110" spans="1:9" ht="15">
@@ -4348,51 +4369,51 @@
         <v>135</v>
       </c>
       <c r="B110" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C110" t="s">
-        <v>144</v>
+        <v>59</v>
       </c>
       <c r="D110" t="s">
-        <v>85</v>
+        <v>56</v>
       </c>
       <c r="E110" t="s">
-        <v>95</v>
+        <v>131</v>
       </c>
       <c r="F110" t="s">
-        <v>158</v>
+        <v>58</v>
       </c>
       <c r="G110" t="s">
-        <v>132</v>
+        <v>28</v>
       </c>
       <c r="H110" t="s">
         <v>18</v>
       </c>
       <c r="I110" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="111" spans="1:9" ht="15">
       <c r="A111" t="s">
+        <v>135</v>
+      </c>
+      <c r="B111" t="s">
+        <v>46</v>
+      </c>
+      <c r="C111" t="s">
+        <v>144</v>
+      </c>
+      <c r="D111" t="s">
+        <v>158</v>
+      </c>
+      <c r="E111" t="s">
+        <v>23</v>
+      </c>
+      <c r="F111" t="s">
         <v>159</v>
       </c>
-      <c r="B111" t="s">
-        <v>20</v>
-      </c>
-      <c r="C111" t="s">
-        <v>21</v>
-      </c>
-      <c r="D111" t="s">
-        <v>22</v>
-      </c>
-      <c r="E111" t="s">
-        <v>27</v>
-      </c>
-      <c r="F111" t="s">
-        <v>16</v>
-      </c>
       <c r="G111" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="H111" t="s">
         <v>18</v>
@@ -4403,74 +4424,74 @@
     </row>
     <row r="112" spans="1:9" ht="15">
       <c r="A112" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="B112" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C112" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D112" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="E112" t="s">
-        <v>92</v>
+        <v>160</v>
       </c>
       <c r="F112" t="s">
-        <v>137</v>
+        <v>104</v>
       </c>
       <c r="G112" t="s">
-        <v>28</v>
+        <v>155</v>
       </c>
       <c r="H112" t="s">
         <v>18</v>
       </c>
       <c r="I112" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="113" spans="1:9" ht="15">
       <c r="A113" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="B113" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="C113" t="s">
-        <v>21</v>
+        <v>144</v>
       </c>
       <c r="D113" t="s">
-        <v>22</v>
+        <v>85</v>
       </c>
       <c r="E113" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="F113" t="s">
-        <v>16</v>
+        <v>161</v>
       </c>
       <c r="G113" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="H113" t="s">
         <v>18</v>
       </c>
       <c r="I113" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="114" spans="1:9" ht="15">
       <c r="A114" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B114" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C114" t="s">
         <v>21</v>
       </c>
       <c r="D114" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E114" t="s">
         <v>27</v>
@@ -4490,22 +4511,22 @@
     </row>
     <row r="115" spans="1:9" ht="15">
       <c r="A115" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B115" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C115" t="s">
         <v>122</v>
       </c>
       <c r="D115" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="E115" t="s">
         <v>92</v>
       </c>
       <c r="F115" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G115" t="s">
         <v>28</v>
@@ -4519,16 +4540,16 @@
     </row>
     <row r="116" spans="1:9" ht="15">
       <c r="A116" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B116" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C116" t="s">
         <v>21</v>
       </c>
       <c r="D116" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E116" t="s">
         <v>27</v>
@@ -4548,25 +4569,25 @@
     </row>
     <row r="117" spans="1:9" ht="15">
       <c r="A117" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B117" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C117" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D117" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E117" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F117" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="G117" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H117" t="s">
         <v>18</v>
@@ -4577,25 +4598,25 @@
     </row>
     <row r="118" spans="1:9" ht="15">
       <c r="A118" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B118" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C118" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D118" t="s">
-        <v>45</v>
+        <v>163</v>
       </c>
       <c r="E118" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F118" t="s">
-        <v>16</v>
+        <v>140</v>
       </c>
       <c r="G118" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H118" t="s">
         <v>18</v>
@@ -4606,25 +4627,25 @@
     </row>
     <row r="119" spans="1:9" ht="15">
       <c r="A119" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B119" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C119" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D119" t="s">
-        <v>161</v>
+        <v>39</v>
       </c>
       <c r="E119" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F119" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="G119" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H119" t="s">
         <v>18</v>
@@ -4635,25 +4656,25 @@
     </row>
     <row r="120" spans="1:9" ht="15">
       <c r="A120" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B120" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C120" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D120" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="E120" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F120" t="s">
-        <v>16</v>
+        <v>140</v>
       </c>
       <c r="G120" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H120" t="s">
         <v>18</v>
@@ -4667,22 +4688,22 @@
         <v>162</v>
       </c>
       <c r="B121" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="C121" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D121" t="s">
         <v>45</v>
       </c>
       <c r="E121" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F121" t="s">
-        <v>124</v>
+        <v>16</v>
       </c>
       <c r="G121" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H121" t="s">
         <v>18</v>
@@ -4696,22 +4717,22 @@
         <v>162</v>
       </c>
       <c r="B122" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C122" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D122" t="s">
-        <v>22</v>
+        <v>164</v>
       </c>
       <c r="E122" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F122" t="s">
-        <v>16</v>
+        <v>140</v>
       </c>
       <c r="G122" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H122" t="s">
         <v>18</v>
@@ -4725,22 +4746,22 @@
         <v>162</v>
       </c>
       <c r="B123" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C123" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D123" t="s">
-        <v>163</v>
+        <v>43</v>
       </c>
       <c r="E123" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F123" t="s">
-        <v>124</v>
+        <v>16</v>
       </c>
       <c r="G123" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H123" t="s">
         <v>18</v>
@@ -4751,25 +4772,25 @@
     </row>
     <row r="124" spans="1:9" ht="15">
       <c r="A124" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B124" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C124" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D124" t="s">
         <v>45</v>
       </c>
       <c r="E124" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F124" t="s">
-        <v>16</v>
+        <v>124</v>
       </c>
       <c r="G124" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H124" t="s">
         <v>18</v>
@@ -4780,25 +4801,25 @@
     </row>
     <row r="125" spans="1:9" ht="15">
       <c r="A125" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B125" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C125" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D125" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E125" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="F125" t="s">
-        <v>124</v>
+        <v>16</v>
       </c>
       <c r="G125" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H125" t="s">
         <v>18</v>
@@ -4809,25 +4830,25 @@
     </row>
     <row r="126" spans="1:9" ht="15">
       <c r="A126" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B126" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C126" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D126" t="s">
-        <v>45</v>
+        <v>166</v>
       </c>
       <c r="E126" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F126" t="s">
-        <v>16</v>
+        <v>124</v>
       </c>
       <c r="G126" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H126" t="s">
         <v>18</v>
@@ -4838,25 +4859,25 @@
     </row>
     <row r="127" spans="1:9" ht="15">
       <c r="A127" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B127" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C127" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D127" t="s">
-        <v>150</v>
+        <v>45</v>
       </c>
       <c r="E127" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F127" t="s">
-        <v>124</v>
+        <v>16</v>
       </c>
       <c r="G127" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H127" t="s">
         <v>18</v>
@@ -4867,25 +4888,25 @@
     </row>
     <row r="128" spans="1:9" ht="15">
       <c r="A128" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B128" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C128" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D128" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E128" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="F128" t="s">
-        <v>16</v>
+        <v>124</v>
       </c>
       <c r="G128" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H128" t="s">
         <v>18</v>
@@ -4896,16 +4917,16 @@
     </row>
     <row r="129" spans="1:9" ht="15">
       <c r="A129" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B129" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C129" t="s">
         <v>21</v>
       </c>
       <c r="D129" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E129" t="s">
         <v>27</v>
@@ -4925,16 +4946,16 @@
     </row>
     <row r="130" spans="1:9" ht="15">
       <c r="A130" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B130" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="C130" t="s">
         <v>122</v>
       </c>
       <c r="D130" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="E130" t="s">
         <v>92</v>
@@ -4954,25 +4975,25 @@
     </row>
     <row r="131" spans="1:9" ht="15">
       <c r="A131" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B131" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="C131" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D131" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="E131" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F131" t="s">
-        <v>124</v>
+        <v>16</v>
       </c>
       <c r="G131" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H131" t="s">
         <v>18</v>
@@ -4983,25 +5004,25 @@
     </row>
     <row r="132" spans="1:9" ht="15">
       <c r="A132" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B132" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C132" t="s">
-        <v>165</v>
+        <v>21</v>
       </c>
       <c r="D132" t="s">
-        <v>166</v>
+        <v>43</v>
       </c>
       <c r="E132" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F132" t="s">
-        <v>167</v>
+        <v>16</v>
       </c>
       <c r="G132" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H132" t="s">
         <v>18</v>
@@ -5012,22 +5033,22 @@
     </row>
     <row r="133" spans="1:9" ht="15">
       <c r="A133" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B133" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C133" t="s">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="D133" t="s">
-        <v>168</v>
+        <v>142</v>
       </c>
       <c r="E133" t="s">
         <v>92</v>
       </c>
       <c r="F133" t="s">
-        <v>167</v>
+        <v>124</v>
       </c>
       <c r="G133" t="s">
         <v>28</v>
@@ -5041,22 +5062,22 @@
     </row>
     <row r="134" spans="1:9" ht="15">
       <c r="A134" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B134" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C134" t="s">
         <v>122</v>
       </c>
       <c r="D134" t="s">
-        <v>130</v>
+        <v>45</v>
       </c>
       <c r="E134" t="s">
         <v>92</v>
       </c>
       <c r="F134" t="s">
-        <v>157</v>
+        <v>124</v>
       </c>
       <c r="G134" t="s">
         <v>28</v>
@@ -5070,22 +5091,22 @@
     </row>
     <row r="135" spans="1:9" ht="15">
       <c r="A135" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B135" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C135" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D135" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E135" t="s">
         <v>92</v>
       </c>
       <c r="F135" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="G135" t="s">
         <v>28</v>
@@ -5099,22 +5120,22 @@
     </row>
     <row r="136" spans="1:9" ht="15">
       <c r="A136" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B136" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C136" t="s">
-        <v>122</v>
+        <v>168</v>
       </c>
       <c r="D136" t="s">
-        <v>123</v>
+        <v>171</v>
       </c>
       <c r="E136" t="s">
         <v>92</v>
       </c>
       <c r="F136" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="G136" t="s">
         <v>28</v>
@@ -5128,22 +5149,22 @@
     </row>
     <row r="137" spans="1:9" ht="15">
       <c r="A137" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B137" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C137" t="s">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="D137" t="s">
-        <v>169</v>
+        <v>130</v>
       </c>
       <c r="E137" t="s">
         <v>92</v>
       </c>
       <c r="F137" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="G137" t="s">
         <v>28</v>
@@ -5157,22 +5178,22 @@
     </row>
     <row r="138" spans="1:9" ht="15">
       <c r="A138" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B138" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C138" t="s">
-        <v>122</v>
+        <v>168</v>
       </c>
       <c r="D138" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="E138" t="s">
         <v>92</v>
       </c>
       <c r="F138" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="G138" t="s">
         <v>28</v>
@@ -5186,22 +5207,22 @@
     </row>
     <row r="139" spans="1:9" ht="15">
       <c r="A139" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B139" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C139" t="s">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="D139" t="s">
-        <v>170</v>
+        <v>123</v>
       </c>
       <c r="E139" t="s">
         <v>92</v>
       </c>
       <c r="F139" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="G139" t="s">
         <v>28</v>
@@ -5215,22 +5236,22 @@
     </row>
     <row r="140" spans="1:9" ht="15">
       <c r="A140" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B140" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C140" t="s">
-        <v>122</v>
+        <v>168</v>
       </c>
       <c r="D140" t="s">
-        <v>123</v>
+        <v>172</v>
       </c>
       <c r="E140" t="s">
         <v>92</v>
       </c>
       <c r="F140" t="s">
-        <v>124</v>
+        <v>170</v>
       </c>
       <c r="G140" t="s">
         <v>28</v>
@@ -5244,22 +5265,22 @@
     </row>
     <row r="141" spans="1:9" ht="15">
       <c r="A141" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B141" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C141" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="D141" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="E141" t="s">
-        <v>173</v>
+        <v>92</v>
       </c>
       <c r="F141" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="G141" t="s">
         <v>28</v>
@@ -5273,22 +5294,22 @@
     </row>
     <row r="142" spans="1:9" ht="15">
       <c r="A142" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B142" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C142" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D142" t="s">
-        <v>106</v>
+        <v>173</v>
       </c>
       <c r="E142" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="F142" t="s">
-        <v>89</v>
+        <v>170</v>
       </c>
       <c r="G142" t="s">
         <v>28</v>
@@ -5302,16 +5323,16 @@
     </row>
     <row r="143" spans="1:9" ht="15">
       <c r="A143" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B143" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C143" t="s">
         <v>122</v>
       </c>
       <c r="D143" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="E143" t="s">
         <v>92</v>
@@ -5331,19 +5352,19 @@
     </row>
     <row r="144" spans="1:9" ht="15">
       <c r="A144" t="s">
+        <v>174</v>
+      </c>
+      <c r="B144" t="s">
+        <v>31</v>
+      </c>
+      <c r="C144" t="s">
+        <v>175</v>
+      </c>
+      <c r="D144" t="s">
         <v>171</v>
       </c>
-      <c r="B144" t="s">
-        <v>38</v>
-      </c>
-      <c r="C144" t="s">
-        <v>172</v>
-      </c>
-      <c r="D144" t="s">
-        <v>168</v>
-      </c>
       <c r="E144" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F144" t="s">
         <v>145</v>
@@ -5360,19 +5381,19 @@
     </row>
     <row r="145" spans="1:9" ht="15">
       <c r="A145" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B145" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C145" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D145" t="s">
-        <v>176</v>
+        <v>106</v>
       </c>
       <c r="E145" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F145" t="s">
         <v>89</v>
@@ -5389,16 +5410,16 @@
     </row>
     <row r="146" spans="1:9" ht="15">
       <c r="A146" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B146" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C146" t="s">
         <v>122</v>
       </c>
       <c r="D146" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="E146" t="s">
         <v>92</v>
@@ -5418,22 +5439,22 @@
     </row>
     <row r="147" spans="1:9" ht="15">
       <c r="A147" t="s">
+        <v>174</v>
+      </c>
+      <c r="B147" t="s">
+        <v>38</v>
+      </c>
+      <c r="C147" t="s">
+        <v>175</v>
+      </c>
+      <c r="D147" t="s">
         <v>171</v>
       </c>
-      <c r="B147" t="s">
-        <v>44</v>
-      </c>
-      <c r="C147" t="s">
-        <v>174</v>
-      </c>
-      <c r="D147" t="s">
-        <v>177</v>
-      </c>
       <c r="E147" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F147" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="G147" t="s">
         <v>28</v>
@@ -5447,22 +5468,22 @@
     </row>
     <row r="148" spans="1:9" ht="15">
       <c r="A148" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B148" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C148" t="s">
-        <v>122</v>
+        <v>177</v>
       </c>
       <c r="D148" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="E148" t="s">
-        <v>92</v>
+        <v>178</v>
       </c>
       <c r="F148" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="G148" t="s">
         <v>28</v>
@@ -5476,22 +5497,22 @@
     </row>
     <row r="149" spans="1:9" ht="15">
       <c r="A149" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B149" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C149" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="D149" t="s">
-        <v>106</v>
+        <v>51</v>
       </c>
       <c r="E149" t="s">
-        <v>178</v>
+        <v>92</v>
       </c>
       <c r="F149" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="G149" t="s">
         <v>28</v>
@@ -5505,19 +5526,19 @@
     </row>
     <row r="150" spans="1:9" ht="15">
       <c r="A150" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B150" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C150" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D150" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E150" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F150" t="s">
         <v>89</v>
@@ -5534,22 +5555,22 @@
     </row>
     <row r="151" spans="1:9" ht="15">
       <c r="A151" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B151" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C151" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
       <c r="D151" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="E151" t="s">
-        <v>178</v>
+        <v>92</v>
       </c>
       <c r="F151" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="G151" t="s">
         <v>28</v>
@@ -5563,22 +5584,22 @@
     </row>
     <row r="152" spans="1:9" ht="15">
       <c r="A152" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B152" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C152" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D152" t="s">
         <v>106</v>
       </c>
       <c r="E152" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F152" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G152" t="s">
         <v>28</v>
@@ -5592,22 +5613,22 @@
     </row>
     <row r="153" spans="1:9" ht="15">
       <c r="A153" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B153" t="s">
-        <v>111</v>
+        <v>46</v>
       </c>
       <c r="C153" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D153" t="s">
-        <v>106</v>
+        <v>179</v>
       </c>
       <c r="E153" t="s">
-        <v>47</v>
+        <v>178</v>
       </c>
       <c r="F153" t="s">
-        <v>154</v>
+        <v>89</v>
       </c>
       <c r="G153" t="s">
         <v>28</v>
@@ -5621,22 +5642,22 @@
     </row>
     <row r="154" spans="1:9" ht="15">
       <c r="A154" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B154" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C154" t="s">
-        <v>122</v>
+        <v>175</v>
       </c>
       <c r="D154" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="E154" t="s">
-        <v>92</v>
+        <v>180</v>
       </c>
       <c r="F154" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="G154" t="s">
         <v>28</v>
@@ -5650,22 +5671,22 @@
     </row>
     <row r="155" spans="1:9" ht="15">
       <c r="A155" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B155" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C155" t="s">
-        <v>122</v>
+        <v>175</v>
       </c>
       <c r="D155" t="s">
-        <v>142</v>
+        <v>106</v>
       </c>
       <c r="E155" t="s">
-        <v>92</v>
+        <v>180</v>
       </c>
       <c r="F155" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="G155" t="s">
         <v>28</v>
@@ -5679,22 +5700,22 @@
     </row>
     <row r="156" spans="1:9" ht="15">
       <c r="A156" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B156" t="s">
-        <v>31</v>
+        <v>111</v>
       </c>
       <c r="C156" t="s">
-        <v>122</v>
+        <v>175</v>
       </c>
       <c r="D156" t="s">
-        <v>51</v>
+        <v>106</v>
       </c>
       <c r="E156" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="F156" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="G156" t="s">
         <v>28</v>
@@ -5708,22 +5729,22 @@
     </row>
     <row r="157" spans="1:9" ht="15">
       <c r="A157" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B157" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="C157" t="s">
         <v>122</v>
       </c>
       <c r="D157" t="s">
-        <v>51</v>
+        <v>139</v>
       </c>
       <c r="E157" t="s">
         <v>92</v>
       </c>
       <c r="F157" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G157" t="s">
         <v>28</v>
@@ -5737,25 +5758,25 @@
     </row>
     <row r="158" spans="1:9" ht="15">
       <c r="A158" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B158" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C158" t="s">
-        <v>180</v>
+        <v>122</v>
       </c>
       <c r="D158" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
       <c r="E158" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F158" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="G158" t="s">
-        <v>133</v>
+        <v>28</v>
       </c>
       <c r="H158" t="s">
         <v>18</v>
@@ -5766,22 +5787,22 @@
     </row>
     <row r="159" spans="1:9" ht="15">
       <c r="A159" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B159" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C159" t="s">
         <v>122</v>
       </c>
       <c r="D159" t="s">
-        <v>152</v>
+        <v>51</v>
       </c>
       <c r="E159" t="s">
         <v>92</v>
       </c>
       <c r="F159" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G159" t="s">
         <v>28</v>
@@ -5795,25 +5816,25 @@
     </row>
     <row r="160" spans="1:9" ht="15">
       <c r="A160" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B160" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C160" t="s">
-        <v>180</v>
+        <v>122</v>
       </c>
       <c r="D160" t="s">
-        <v>169</v>
+        <v>51</v>
       </c>
       <c r="E160" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F160" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="G160" t="s">
-        <v>133</v>
+        <v>28</v>
       </c>
       <c r="H160" t="s">
         <v>18</v>
@@ -5824,25 +5845,25 @@
     </row>
     <row r="161" spans="1:9" ht="15">
       <c r="A161" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B161" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C161" t="s">
-        <v>122</v>
+        <v>182</v>
       </c>
       <c r="D161" t="s">
-        <v>96</v>
+        <v>172</v>
       </c>
       <c r="E161" t="s">
-        <v>92</v>
+        <v>27</v>
       </c>
       <c r="F161" t="s">
-        <v>137</v>
+        <v>41</v>
       </c>
       <c r="G161" t="s">
-        <v>28</v>
+        <v>133</v>
       </c>
       <c r="H161" t="s">
         <v>18</v>
@@ -5853,25 +5874,25 @@
     </row>
     <row r="162" spans="1:9" ht="15">
       <c r="A162" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B162" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C162" t="s">
-        <v>180</v>
+        <v>122</v>
       </c>
       <c r="D162" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E162" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F162" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="G162" t="s">
-        <v>133</v>
+        <v>28</v>
       </c>
       <c r="H162" t="s">
         <v>18</v>
@@ -5882,16 +5903,16 @@
     </row>
     <row r="163" spans="1:9" ht="15">
       <c r="A163" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B163" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C163" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D163" t="s">
-        <v>150</v>
+        <v>172</v>
       </c>
       <c r="E163" t="s">
         <v>27</v>
@@ -5911,25 +5932,25 @@
     </row>
     <row r="164" spans="1:9" ht="15">
       <c r="A164" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B164" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C164" t="s">
-        <v>180</v>
+        <v>122</v>
       </c>
       <c r="D164" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="E164" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="F164" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="G164" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="H164" t="s">
         <v>18</v>
@@ -5943,22 +5964,22 @@
         <v>181</v>
       </c>
       <c r="B165" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C165" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D165" t="s">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="E165" t="s">
-        <v>175</v>
+        <v>27</v>
       </c>
       <c r="F165" t="s">
-        <v>89</v>
+        <v>41</v>
       </c>
       <c r="G165" t="s">
-        <v>28</v>
+        <v>133</v>
       </c>
       <c r="H165" t="s">
         <v>18</v>
@@ -5972,22 +5993,22 @@
         <v>181</v>
       </c>
       <c r="B166" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C166" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D166" t="s">
-        <v>184</v>
+        <v>150</v>
       </c>
       <c r="E166" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="F166" t="s">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="G166" t="s">
-        <v>28</v>
+        <v>133</v>
       </c>
       <c r="H166" t="s">
         <v>18</v>
@@ -6001,22 +6022,22 @@
         <v>181</v>
       </c>
       <c r="B167" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="C167" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D167" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="E167" t="s">
-        <v>175</v>
+        <v>27</v>
       </c>
       <c r="F167" t="s">
-        <v>89</v>
+        <v>41</v>
       </c>
       <c r="G167" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="H167" t="s">
         <v>18</v>
@@ -6027,22 +6048,22 @@
     </row>
     <row r="168" spans="1:9" ht="15">
       <c r="A168" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B168" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="C168" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D168" t="s">
-        <v>116</v>
+        <v>184</v>
       </c>
       <c r="E168" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="F168" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G168" t="s">
         <v>28</v>
@@ -6056,16 +6077,16 @@
     </row>
     <row r="169" spans="1:9" ht="15">
       <c r="A169" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B169" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C169" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D169" t="s">
-        <v>45</v>
+        <v>186</v>
       </c>
       <c r="E169" t="s">
         <v>63</v>
@@ -6085,19 +6106,19 @@
     </row>
     <row r="170" spans="1:9" ht="15">
       <c r="A170" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B170" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C170" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D170" t="s">
-        <v>114</v>
+        <v>45</v>
       </c>
       <c r="E170" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F170" t="s">
         <v>89</v>
@@ -6114,16 +6135,16 @@
     </row>
     <row r="171" spans="1:9" ht="15">
       <c r="A171" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B171" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C171" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D171" t="s">
-        <v>45</v>
+        <v>116</v>
       </c>
       <c r="E171" t="s">
         <v>63</v>
@@ -6143,22 +6164,22 @@
     </row>
     <row r="172" spans="1:9" ht="15">
       <c r="A172" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B172" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C172" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D172" t="s">
-        <v>185</v>
+        <v>45</v>
       </c>
       <c r="E172" t="s">
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="F172" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G172" t="s">
         <v>28</v>
@@ -6172,22 +6193,22 @@
     </row>
     <row r="173" spans="1:9" ht="15">
       <c r="A173" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B173" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C173" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D173" t="s">
-        <v>156</v>
+        <v>114</v>
       </c>
       <c r="E173" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="F173" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G173" t="s">
         <v>28</v>
@@ -6201,22 +6222,22 @@
     </row>
     <row r="174" spans="1:9" ht="15">
       <c r="A174" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B174" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C174" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D174" t="s">
-        <v>116</v>
+        <v>45</v>
       </c>
       <c r="E174" t="s">
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="F174" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G174" t="s">
         <v>28</v>
@@ -6230,22 +6251,22 @@
     </row>
     <row r="175" spans="1:9" ht="15">
       <c r="A175" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B175" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C175" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D175" t="s">
-        <v>140</v>
+        <v>187</v>
       </c>
       <c r="E175" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="F175" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G175" t="s">
         <v>28</v>
@@ -6259,22 +6280,22 @@
     </row>
     <row r="176" spans="1:9" ht="15">
       <c r="A176" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B176" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C176" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D176" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="E176" t="s">
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="F176" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G176" t="s">
         <v>28</v>
@@ -6288,22 +6309,22 @@
     </row>
     <row r="177" spans="1:9" ht="15">
       <c r="A177" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B177" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C177" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D177" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="E177" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="F177" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G177" t="s">
         <v>28</v>
@@ -6317,22 +6338,22 @@
     </row>
     <row r="178" spans="1:9" ht="15">
       <c r="A178" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B178" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C178" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D178" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
       <c r="E178" t="s">
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="F178" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G178" t="s">
         <v>28</v>
@@ -6346,22 +6367,22 @@
     </row>
     <row r="179" spans="1:9" ht="15">
       <c r="A179" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B179" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C179" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D179" t="s">
-        <v>106</v>
+        <v>154</v>
       </c>
       <c r="E179" t="s">
-        <v>63</v>
+        <v>178</v>
       </c>
       <c r="F179" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G179" t="s">
         <v>28</v>
@@ -6375,22 +6396,22 @@
     </row>
     <row r="180" spans="1:9" ht="15">
       <c r="A180" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B180" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C180" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D180" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="E180" t="s">
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="F180" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G180" t="s">
         <v>28</v>
@@ -6399,6 +6420,93 @@
         <v>18</v>
       </c>
       <c r="I180" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" ht="15">
+      <c r="A181" t="s">
+        <v>183</v>
+      </c>
+      <c r="B181" t="s">
+        <v>49</v>
+      </c>
+      <c r="C181" t="s">
+        <v>177</v>
+      </c>
+      <c r="D181" t="s">
+        <v>157</v>
+      </c>
+      <c r="E181" t="s">
+        <v>178</v>
+      </c>
+      <c r="F181" t="s">
+        <v>89</v>
+      </c>
+      <c r="G181" t="s">
+        <v>28</v>
+      </c>
+      <c r="H181" t="s">
+        <v>18</v>
+      </c>
+      <c r="I181" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" ht="15">
+      <c r="A182" t="s">
+        <v>183</v>
+      </c>
+      <c r="B182" t="s">
+        <v>55</v>
+      </c>
+      <c r="C182" t="s">
+        <v>185</v>
+      </c>
+      <c r="D182" t="s">
+        <v>106</v>
+      </c>
+      <c r="E182" t="s">
+        <v>63</v>
+      </c>
+      <c r="F182" t="s">
+        <v>93</v>
+      </c>
+      <c r="G182" t="s">
+        <v>28</v>
+      </c>
+      <c r="H182" t="s">
+        <v>18</v>
+      </c>
+      <c r="I182" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" ht="15">
+      <c r="A183" t="s">
+        <v>183</v>
+      </c>
+      <c r="B183" t="s">
+        <v>55</v>
+      </c>
+      <c r="C183" t="s">
+        <v>177</v>
+      </c>
+      <c r="D183" t="s">
+        <v>85</v>
+      </c>
+      <c r="E183" t="s">
+        <v>178</v>
+      </c>
+      <c r="F183" t="s">
+        <v>89</v>
+      </c>
+      <c r="G183" t="s">
+        <v>28</v>
+      </c>
+      <c r="H183" t="s">
+        <v>18</v>
+      </c>
+      <c r="I183" t="s">
         <v>29</v>
       </c>
     </row>
@@ -6410,15 +6518,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{6a8900d8-3782-4001-9da3-cfb534853d23}">
-  <dimension ref="A1:I8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d569cde3-c7c6-4a19-b502-290fab4762fc}">
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
     <col min="2" max="2" width="11.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="22.8571428571429" customWidth="1"/>
     <col min="4" max="4" width="42.2857142857143" customWidth="1"/>
-    <col min="5" max="5" width="25.8571428571429" customWidth="1"/>
+    <col min="5" max="5" width="26.5714285714286" customWidth="1"/>
     <col min="6" max="6" width="7.42857142857143" customWidth="1"/>
     <col min="7" max="7" width="45.5714285714286" customWidth="1"/>
     <col min="8" max="8" width="9.28571428571429" customWidth="1"/>
@@ -6430,16 +6538,16 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
@@ -6459,13 +6567,13 @@
         <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E2" t="s">
         <v>27</v>
@@ -6488,19 +6596,19 @@
         <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G3" t="s">
         <v>76</v>
@@ -6517,13 +6625,13 @@
         <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E4" t="s">
         <v>27</v>
@@ -6546,19 +6654,19 @@
         <v>135</v>
       </c>
       <c r="B5" t="s">
+        <v>200</v>
+      </c>
+      <c r="C5" t="s">
+        <v>201</v>
+      </c>
+      <c r="D5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F5" t="s">
         <v>198</v>
-      </c>
-      <c r="C5" t="s">
-        <v>199</v>
-      </c>
-      <c r="D5" t="s">
-        <v>200</v>
-      </c>
-      <c r="E5" t="s">
-        <v>201</v>
-      </c>
-      <c r="F5" t="s">
-        <v>196</v>
       </c>
       <c r="G5" t="s">
         <v>113</v>
@@ -6572,25 +6680,25 @@
     </row>
     <row r="6" spans="1:9" ht="15">
       <c r="A6" t="s">
-        <v>162</v>
+        <v>135</v>
       </c>
       <c r="B6" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>205</v>
       </c>
       <c r="D6" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>207</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>198</v>
       </c>
       <c r="G6" t="s">
-        <v>29</v>
+        <v>113</v>
       </c>
       <c r="H6" t="s">
         <v>18</v>
@@ -6601,16 +6709,16 @@
     </row>
     <row r="7" spans="1:9" ht="15">
       <c r="A7" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E7" t="s">
         <v>27</v>
@@ -6630,30 +6738,59 @@
     </row>
     <row r="8" spans="1:9" ht="15">
       <c r="A8" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="B8" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15">
+      <c r="A9" t="s">
         <v>183</v>
       </c>
-      <c r="D8" t="s">
-        <v>191</v>
-      </c>
-      <c r="E8" t="s">
-        <v>202</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="B9" t="s">
+        <v>192</v>
+      </c>
+      <c r="C9" t="s">
+        <v>185</v>
+      </c>
+      <c r="D9" t="s">
+        <v>193</v>
+      </c>
+      <c r="E9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F9" t="s">
         <v>93</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G9" t="s">
         <v>28</v>
       </c>
-      <c r="H8" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="H9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" t="s">
         <v>29</v>
       </c>
     </row>
@@ -6665,8 +6802,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{df5b2c11-046a-496e-8074-d14a98b5a2fa}">
-  <dimension ref="A1:F31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f5ed6959-bd6f-46dd-8e1f-815ee48c626e}">
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
@@ -6682,13 +6819,13 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -6702,16 +6839,16 @@
         <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C2" t="s">
         <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="E2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="F2" t="s">
         <v>18</v>
@@ -6722,13 +6859,13 @@
         <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C3" t="s">
         <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="E3" t="s">
         <v>42</v>
@@ -6742,13 +6879,13 @@
         <v>112</v>
       </c>
       <c r="B4" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E4" t="s">
         <v>80</v>
@@ -6762,13 +6899,13 @@
         <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C5" t="s">
         <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="E5" t="s">
         <v>90</v>
@@ -6782,16 +6919,16 @@
         <v>118</v>
       </c>
       <c r="B6" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E6" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="F6" t="s">
         <v>18</v>
@@ -6802,13 +6939,13 @@
         <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="E7" t="s">
         <v>17</v>
@@ -6822,16 +6959,16 @@
         <v>118</v>
       </c>
       <c r="B8" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C8" t="s">
         <v>122</v>
       </c>
       <c r="D8" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E8" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F8" t="s">
         <v>18</v>
@@ -6842,16 +6979,16 @@
         <v>135</v>
       </c>
       <c r="B9" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="C9" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D9" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E9" t="s">
-        <v>213</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
         <v>18</v>
@@ -6862,16 +6999,16 @@
         <v>135</v>
       </c>
       <c r="B10" t="s">
-        <v>204</v>
+        <v>222</v>
       </c>
       <c r="C10" t="s">
         <v>122</v>
       </c>
       <c r="D10" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E10" t="s">
-        <v>146</v>
+        <v>219</v>
       </c>
       <c r="F10" t="s">
         <v>18</v>
@@ -6882,16 +7019,16 @@
         <v>135</v>
       </c>
       <c r="B11" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="D11" t="s">
         <v>216</v>
       </c>
       <c r="E11" t="s">
-        <v>217</v>
+        <v>146</v>
       </c>
       <c r="F11" t="s">
         <v>18</v>
@@ -6902,16 +7039,16 @@
         <v>135</v>
       </c>
       <c r="B12" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="E12" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="F12" t="s">
         <v>18</v>
@@ -6922,16 +7059,16 @@
         <v>135</v>
       </c>
       <c r="B13" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="E13" t="s">
-        <v>138</v>
+        <v>225</v>
       </c>
       <c r="F13" t="s">
         <v>18</v>
@@ -6942,16 +7079,16 @@
         <v>135</v>
       </c>
       <c r="B14" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C14" t="s">
-        <v>144</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>205</v>
+        <v>226</v>
       </c>
       <c r="E14" t="s">
-        <v>42</v>
+        <v>141</v>
       </c>
       <c r="F14" t="s">
         <v>18</v>
@@ -6962,16 +7099,16 @@
         <v>135</v>
       </c>
       <c r="B15" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="D15" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="F15" t="s">
         <v>18</v>
@@ -6982,16 +7119,16 @@
         <v>135</v>
       </c>
       <c r="B16" t="s">
+        <v>213</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
         <v>214</v>
       </c>
-      <c r="C16" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" t="s">
-        <v>219</v>
-      </c>
       <c r="E16" t="s">
-        <v>132</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
@@ -7005,13 +7142,13 @@
         <v>220</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="D17" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="E17" t="s">
-        <v>80</v>
+        <v>132</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -7022,16 +7159,16 @@
         <v>135</v>
       </c>
       <c r="B18" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="C18" t="s">
-        <v>222</v>
+        <v>21</v>
       </c>
       <c r="D18" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E18" t="s">
-        <v>223</v>
+        <v>80</v>
       </c>
       <c r="F18" t="s">
         <v>18</v>
@@ -7039,19 +7176,19 @@
     </row>
     <row r="19" spans="1:6" ht="15">
       <c r="A19" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
       <c r="C19" t="s">
-        <v>122</v>
+        <v>229</v>
       </c>
       <c r="D19" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>230</v>
       </c>
       <c r="F19" t="s">
         <v>18</v>
@@ -7059,16 +7196,16 @@
     </row>
     <row r="20" spans="1:6" ht="15">
       <c r="A20" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C20" t="s">
         <v>122</v>
       </c>
       <c r="D20" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E20" t="s">
         <v>29</v>
@@ -7082,7 +7219,7 @@
         <v>162</v>
       </c>
       <c r="B21" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C21" t="s">
         <v>122</v>
@@ -7099,16 +7236,16 @@
     </row>
     <row r="22" spans="1:6" ht="15">
       <c r="A22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B22" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="C22" t="s">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="D22" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
@@ -7119,16 +7256,16 @@
     </row>
     <row r="23" spans="1:6" ht="15">
       <c r="A23" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B23" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="C23" t="s">
-        <v>122</v>
+        <v>168</v>
       </c>
       <c r="D23" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="E23" t="s">
         <v>29</v>
@@ -7139,16 +7276,16 @@
     </row>
     <row r="24" spans="1:6" ht="15">
       <c r="A24" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B24" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C24" t="s">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="D24" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E24" t="s">
         <v>29</v>
@@ -7159,16 +7296,16 @@
     </row>
     <row r="25" spans="1:6" ht="15">
       <c r="A25" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="C25" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D25" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -7179,16 +7316,16 @@
     </row>
     <row r="26" spans="1:6" ht="15">
       <c r="A26" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B26" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="C26" t="s">
-        <v>122</v>
+        <v>168</v>
       </c>
       <c r="D26" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="E26" t="s">
         <v>29</v>
@@ -7199,16 +7336,16 @@
     </row>
     <row r="27" spans="1:6" ht="15">
       <c r="A27" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B27" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C27" t="s">
         <v>122</v>
       </c>
       <c r="D27" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E27" t="s">
         <v>29</v>
@@ -7219,16 +7356,16 @@
     </row>
     <row r="28" spans="1:6" ht="15">
       <c r="A28" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B28" t="s">
-        <v>204</v>
+        <v>222</v>
       </c>
       <c r="C28" t="s">
         <v>122</v>
       </c>
       <c r="D28" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E28" t="s">
         <v>29</v>
@@ -7242,13 +7379,13 @@
         <v>181</v>
       </c>
       <c r="B29" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C29" t="s">
-        <v>174</v>
+        <v>122</v>
       </c>
       <c r="D29" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="E29" t="s">
         <v>29</v>
@@ -7259,16 +7396,16 @@
     </row>
     <row r="30" spans="1:6" ht="15">
       <c r="A30" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B30" t="s">
+        <v>215</v>
+      </c>
+      <c r="C30" t="s">
+        <v>177</v>
+      </c>
+      <c r="D30" t="s">
         <v>211</v>
-      </c>
-      <c r="C30" t="s">
-        <v>183</v>
-      </c>
-      <c r="D30" t="s">
-        <v>216</v>
       </c>
       <c r="E30" t="s">
         <v>29</v>
@@ -7279,21 +7416,41 @@
     </row>
     <row r="31" spans="1:6" ht="15">
       <c r="A31" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B31" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="C31" t="s">
+        <v>185</v>
+      </c>
+      <c r="D31" t="s">
+        <v>223</v>
+      </c>
+      <c r="E31" t="s">
+        <v>29</v>
+      </c>
+      <c r="F31" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="15">
+      <c r="A32" t="s">
         <v>183</v>
       </c>
-      <c r="D31" t="s">
-        <v>216</v>
-      </c>
-      <c r="E31" t="s">
-        <v>29</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="B32" t="s">
+        <v>231</v>
+      </c>
+      <c r="C32" t="s">
+        <v>185</v>
+      </c>
+      <c r="D32" t="s">
+        <v>223</v>
+      </c>
+      <c r="E32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F32" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nie publikuj wpisów nauczania indywidualnego (IND)
Nauczanie indywidualne dotyczy jednego ucznia z imienia i nazwiska, więc
nie ma go na żadnej ze stron. Eksport oznacza je dwojako: przedrostkiem
w kolumnie "Oddział" (4TFB|IND*KM) i w nazwie dziennika zajęć innych
(IN - Nazwisko Imię [klasa]).

Sanitizer zostawia teraz dziennikom IND sam znacznik "IND" zamiast pustej
komórki — dane ucznia nadal znikają, ale generator widzi kategorię i może
wiersz pominąć. Bez tego filtr byłby niemożliwy po oczyszczeniu pliku.

W tej paczce odpada 1 zastępstwo (4TFB|IND*KM, 23.09 lekcja 5) i wszystkie
5 zajęć innych, więc sekcja zajęć innych jest pusta — to poprawny wynik,
nie błąd odczytu.

Dopasowanie jest dosłowne (^IND?\b), więc INFORMATYKA ani "Indywidualny
tok" się nie łapią.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOZastepstwach.xlsx
+++ b/InformacjeOZastepstwach.xlsx
@@ -429,7 +429,7 @@
     <s:t>17:25-18:10</s:t>
   </s:si>
   <s:si>
-    <s:t/>
+    <s:t>IND</s:t>
   </s:si>
   <s:si>
     <s:t xml:space="preserve">Matematyka </s:t>
@@ -438,7 +438,7 @@
     <s:t>08:00-08:45</s:t>
   </s:si>
   <s:si>
-    <s:t/>
+    <s:t>IND</s:t>
   </s:si>
   <s:si>
     <s:t>08:50-09:35</s:t>

</xml_diff>

<commit_message>
Popraw zastępstwo 2TFA 23.09: biblioteka zamiast języka polskiego
Korekta zgłoszona przez użytkownika. Lekcja 5 (informatyka, Maciej Najwer)
ma zastępstwo Barbary Wrzeszcz — zajęcia biblioteczne w bibliotece, a nie
język polski u Magdaleny Ulanowskiej.

Sala i przedmiot zapisane konwencją eksportu ("Zajęcia biblioteczne",
sala "bib"), forma płatności ustawiona na "Bezpłatne" — tak ma każdy inny
wpis biblioteczny Barbary Wrzeszcz w tej paczce.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOZastepstwach.xlsx
+++ b/InformacjeOZastepstwach.xlsx
@@ -580,7 +580,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>-</t>
@@ -623,7 +622,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -713,7 +711,6 @@
           <t>Filipiak Wiesław</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -756,7 +753,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -799,7 +795,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -842,7 +837,6 @@
           <t>Filipiak Wiesław</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -885,7 +879,6 @@
           <t>Kaczorowski Waldemar</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -928,7 +921,6 @@
           <t>Granatowska Mariola</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -971,7 +963,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1014,7 +1005,6 @@
           <t>Nowak Magdalena</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1057,7 +1047,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -1100,7 +1089,6 @@
           <t>Galert Anna</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1143,7 +1131,6 @@
           <t>Wojciechowski Łukasz</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -1186,7 +1173,6 @@
           <t>Filipek Anna</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1229,7 +1215,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1272,7 +1257,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>-</t>
@@ -1315,7 +1299,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>-</t>
@@ -1358,7 +1341,6 @@
           <t>Zając Ewa</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -1401,7 +1383,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>-</t>
@@ -1444,7 +1425,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1487,7 +1467,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>-</t>
@@ -1530,7 +1509,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>-</t>
@@ -1573,7 +1551,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1616,7 +1593,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>-</t>
@@ -1659,7 +1635,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>-</t>
@@ -1702,7 +1677,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1745,7 +1719,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1788,7 +1761,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1831,7 +1803,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1874,7 +1845,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>-</t>
@@ -1917,7 +1887,6 @@
           <t>Leńczowska Iwona</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1960,7 +1929,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>-</t>
@@ -2003,7 +1971,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2046,7 +2013,6 @@
           <t>Wojciechowski Łukasz</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2089,7 +2055,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>-</t>
@@ -2132,7 +2097,6 @@
           <t>Zając Ewa</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2222,7 +2186,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2265,7 +2228,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>-</t>
@@ -2308,7 +2270,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2351,7 +2312,6 @@
           <t>Sałdyka Karolina</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2394,7 +2354,6 @@
           <t>Zając Ewa</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -2437,7 +2396,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>-</t>
@@ -2480,7 +2438,6 @@
           <t>Płatek Krzysztof</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2570,7 +2527,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2613,7 +2569,6 @@
           <t>Płatek Krzysztof</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2656,7 +2611,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>-</t>
@@ -2699,7 +2653,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>-</t>
@@ -2742,7 +2695,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>-</t>
@@ -2785,7 +2737,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>-</t>
@@ -2828,7 +2779,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2871,7 +2821,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>-</t>
@@ -2914,7 +2863,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>-</t>
@@ -2957,7 +2905,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3000,7 +2947,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>-</t>
@@ -3043,7 +2989,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>-</t>
@@ -3086,7 +3031,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3176,7 +3120,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -3219,7 +3162,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>-</t>
@@ -3262,7 +3204,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3305,7 +3246,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3348,7 +3288,6 @@
           <t>Wojciechowski Łukasz</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3391,7 +3330,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>-</t>
@@ -3434,7 +3372,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3477,7 +3414,6 @@
           <t>Nestoruk Lidia</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3520,7 +3456,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3563,7 +3498,6 @@
           <t>Kruk Marcin</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3593,23 +3527,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Język polski</t>
+          <t>Zajęcia biblioteczne</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>bib</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Ulanowska Magdalena</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr"/>
+          <t>Wrzeszcz Barbara</t>
+        </is>
+      </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Dodatkowo płatne</t>
+          <t>Bezpłatne</t>
         </is>
       </c>
     </row>
@@ -3639,13 +3572,11 @@
           <t>Język polski</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
           <t>-</t>
@@ -3688,7 +3619,6 @@
           <t>Krzemińska Beata</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3731,7 +3661,6 @@
           <t>Nestoruk Lidia</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3774,7 +3703,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3817,7 +3745,6 @@
           <t>Mucha Anna</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3860,7 +3787,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
           <t>-</t>
@@ -3903,7 +3829,6 @@
           <t>Galert Anna</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3946,7 +3871,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr">
         <is>
           <t>-</t>
@@ -3989,7 +3913,6 @@
           <t>Misiąg Anna</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -4032,7 +3955,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
         <is>
           <t>-</t>
@@ -4075,7 +3997,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
           <t>-</t>
@@ -4118,7 +4039,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr">
         <is>
           <t>-</t>
@@ -4161,7 +4081,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
           <t>-</t>
@@ -4204,7 +4123,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
           <t>-</t>
@@ -4247,7 +4165,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
           <t>-</t>
@@ -4290,7 +4207,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr">
         <is>
           <t>-</t>
@@ -4333,7 +4249,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
           <t>-</t>
@@ -4376,7 +4291,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr">
         <is>
           <t>-</t>
@@ -4419,7 +4333,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
           <t>-</t>
@@ -4462,7 +4375,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
       <c r="I92" t="inlineStr">
         <is>
           <t>-</t>
@@ -4505,7 +4417,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
           <t>-</t>
@@ -4548,7 +4459,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr">
         <is>
           <t>-</t>
@@ -4591,7 +4501,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
           <t>-</t>
@@ -4634,7 +4543,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr">
         <is>
           <t>-</t>
@@ -4677,7 +4585,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
           <t>-</t>
@@ -4720,7 +4627,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr">
         <is>
           <t>-</t>
@@ -4763,7 +4669,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
           <t>-</t>
@@ -4806,7 +4711,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr">
         <is>
           <t>-</t>
@@ -4849,7 +4753,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
           <t>-</t>
@@ -4892,7 +4795,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
           <t>-</t>
@@ -4935,7 +4837,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
           <t>-</t>
@@ -4978,7 +4879,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr">
         <is>
           <t>-</t>
@@ -5021,7 +4921,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>-</t>
@@ -5064,7 +4963,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
           <t>-</t>
@@ -5107,7 +5005,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>-</t>
@@ -5150,7 +5047,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr">
         <is>
           <t>-</t>
@@ -5193,7 +5089,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
           <t>-</t>
@@ -5236,7 +5131,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr">
         <is>
           <t>-</t>
@@ -5279,7 +5173,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
           <t>-</t>
@@ -5322,7 +5215,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr">
         <is>
           <t>-</t>
@@ -5365,7 +5257,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
           <t>-</t>
@@ -5408,7 +5299,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
           <t>-</t>
@@ -5451,7 +5341,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
           <t>-</t>
@@ -5494,7 +5383,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
           <t>-</t>
@@ -5537,7 +5425,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
           <t>-</t>
@@ -5580,7 +5467,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
           <t>-</t>
@@ -5623,7 +5509,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
           <t>-</t>
@@ -5666,7 +5551,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
           <t>-</t>
@@ -5709,7 +5593,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>-</t>
@@ -5752,7 +5635,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
           <t>-</t>
@@ -5795,7 +5677,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>-</t>
@@ -5838,7 +5719,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
           <t>-</t>
@@ -5881,7 +5761,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>-</t>
@@ -5924,7 +5803,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>-</t>
@@ -5967,7 +5845,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
           <t>-</t>
@@ -6010,7 +5887,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr">
         <is>
           <t>-</t>
@@ -6053,7 +5929,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
           <t>-</t>
@@ -6096,7 +5971,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
       <c r="I130" t="inlineStr">
         <is>
           <t>-</t>
@@ -6139,7 +6013,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
           <t>-</t>
@@ -6182,7 +6055,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
       <c r="I132" t="inlineStr">
         <is>
           <t>-</t>
@@ -6225,7 +6097,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
           <t>-</t>
@@ -6268,7 +6139,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr">
         <is>
           <t>-</t>
@@ -6311,7 +6181,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
           <t>-</t>
@@ -6354,7 +6223,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
       <c r="I136" t="inlineStr">
         <is>
           <t>-</t>
@@ -6397,7 +6265,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
           <t>-</t>
@@ -6440,7 +6307,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
       <c r="I138" t="inlineStr">
         <is>
           <t>-</t>
@@ -6483,7 +6349,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
           <t>-</t>
@@ -6526,7 +6391,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
       <c r="I140" t="inlineStr">
         <is>
           <t>-</t>
@@ -6569,7 +6433,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
           <t>-</t>
@@ -6612,7 +6475,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
       <c r="I142" t="inlineStr">
         <is>
           <t>-</t>
@@ -6655,7 +6517,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
           <t>-</t>
@@ -6698,7 +6559,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
       <c r="I144" t="inlineStr">
         <is>
           <t>-</t>
@@ -6741,7 +6601,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
           <t>-</t>
@@ -6784,7 +6643,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
       <c r="I146" t="inlineStr">
         <is>
           <t>-</t>
@@ -6827,7 +6685,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
           <t>-</t>
@@ -6870,7 +6727,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
       <c r="I148" t="inlineStr">
         <is>
           <t>-</t>
@@ -6987,7 +6843,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>-</t>
@@ -7030,7 +6885,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>-</t>
@@ -7073,7 +6927,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>-</t>
@@ -7106,13 +6959,11 @@
           <t>język polski</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>-</t>
@@ -7155,7 +7006,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>-</t>
@@ -7244,7 +7094,6 @@
           <t>Ostrowska Ewa</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -7272,7 +7121,6 @@
           <t>Kosin Anna</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -7300,7 +7148,6 @@
           <t>Małecka Barbara</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -7328,7 +7175,6 @@
           <t>Mucha Anna</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -7356,7 +7202,6 @@
           <t>Skarupa Agnieszka</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -7384,7 +7229,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -7412,7 +7256,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -7440,7 +7283,6 @@
           <t>Misiąg Anna</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -7468,7 +7310,6 @@
           <t>Ulanowska Magdalena</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -7496,7 +7337,6 @@
           <t>Socha Dariusz</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -7524,7 +7364,6 @@
           <t>Cieśla Marcin</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -7552,7 +7391,6 @@
           <t>Małecka Barbara</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -7580,7 +7418,6 @@
           <t>Kruk Marcin</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" t="inlineStr">
@@ -7608,7 +7445,6 @@
           <t>Krycia Ewelina</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" t="inlineStr">
@@ -7636,7 +7472,6 @@
           <t>Danielewski Paweł</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -7664,7 +7499,6 @@
           <t>Skarupa Agnieszka</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -7692,7 +7526,6 @@
           <t>Zaleska Magdalena</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" t="inlineStr">
@@ -7720,7 +7553,6 @@
           <t>Krzemińska Beata</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" t="inlineStr">
@@ -7748,7 +7580,6 @@
           <t>Płatek Krzysztof</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -7776,7 +7607,6 @@
           <t>Smirnow-Zechman Eleonora</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" t="inlineStr">
@@ -7804,7 +7634,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" t="inlineStr">
@@ -7832,7 +7661,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" t="inlineStr">
@@ -7860,7 +7688,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" t="inlineStr">
@@ -7888,7 +7715,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" t="inlineStr">
@@ -7916,7 +7742,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" t="inlineStr">
@@ -7944,7 +7769,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" t="inlineStr">
@@ -7972,7 +7796,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" t="inlineStr">
@@ -8000,7 +7823,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" t="inlineStr">
@@ -8028,7 +7850,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" t="inlineStr">
@@ -8056,7 +7877,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8084,7 +7904,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8112,7 +7931,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8140,7 +7958,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8168,7 +7985,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>

<commit_message>
Popraw zastępstwo 1TFH 25.09 l.4: Smirnow-Zechman, biznes i zarządzanie
Korekta zgłoszona przez użytkownika. Za Magdalenę Nowak lekcję 4
(10:35-11:20) prowadzi Eleonora Smirnow-Zechman — biznes i zarządzanie
w sali 22 — a nie Waldemar Kaczorowski z historią. Forma płatności bez
zmian ("Dodatkowo płatne").

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOZastepstwach.xlsx
+++ b/InformacjeOZastepstwach.xlsx
@@ -580,7 +580,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>-</t>
@@ -623,7 +622,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -713,7 +711,6 @@
           <t>Filipiak Wiesław</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -756,7 +753,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -799,7 +795,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -842,7 +837,6 @@
           <t>Filipiak Wiesław</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -885,7 +879,6 @@
           <t>Kaczorowski Waldemar</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -928,7 +921,6 @@
           <t>Granatowska Mariola</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -971,7 +963,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1014,7 +1005,6 @@
           <t>Nowak Magdalena</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1057,7 +1047,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -1100,7 +1089,6 @@
           <t>Galert Anna</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1143,7 +1131,6 @@
           <t>Wojciechowski Łukasz</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -1186,7 +1173,6 @@
           <t>Filipek Anna</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1229,7 +1215,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1272,7 +1257,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>-</t>
@@ -1315,7 +1299,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>-</t>
@@ -1358,7 +1341,6 @@
           <t>Zając Ewa</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -1401,7 +1383,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>-</t>
@@ -1444,7 +1425,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1487,7 +1467,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>-</t>
@@ -1530,7 +1509,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>-</t>
@@ -1573,7 +1551,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1616,7 +1593,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>-</t>
@@ -1659,7 +1635,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>-</t>
@@ -1702,7 +1677,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1745,7 +1719,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1788,7 +1761,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1831,7 +1803,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1874,7 +1845,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>-</t>
@@ -1917,7 +1887,6 @@
           <t>Leńczowska Iwona</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -1960,7 +1929,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>-</t>
@@ -2003,7 +1971,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2046,7 +2013,6 @@
           <t>Wojciechowski Łukasz</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2089,7 +2055,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>-</t>
@@ -2132,7 +2097,6 @@
           <t>Zając Ewa</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2222,7 +2186,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2265,7 +2228,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>-</t>
@@ -2308,7 +2270,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2351,7 +2312,6 @@
           <t>Sałdyka Karolina</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2394,7 +2354,6 @@
           <t>Zając Ewa</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -2437,7 +2396,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>-</t>
@@ -2480,7 +2438,6 @@
           <t>Płatek Krzysztof</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2570,7 +2527,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2613,7 +2569,6 @@
           <t>Płatek Krzysztof</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2656,7 +2611,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>-</t>
@@ -2699,7 +2653,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>-</t>
@@ -2742,7 +2695,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>-</t>
@@ -2785,7 +2737,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>-</t>
@@ -2828,7 +2779,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -2871,7 +2821,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>-</t>
@@ -2914,7 +2863,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>-</t>
@@ -2957,7 +2905,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3000,7 +2947,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>-</t>
@@ -3043,7 +2989,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>-</t>
@@ -3086,7 +3031,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3176,7 +3120,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -3219,7 +3162,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>-</t>
@@ -3262,7 +3204,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3305,7 +3246,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3348,7 +3288,6 @@
           <t>Wojciechowski Łukasz</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3391,7 +3330,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>-</t>
@@ -3434,7 +3372,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3477,7 +3414,6 @@
           <t>Nestoruk Lidia</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3520,7 +3456,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3563,7 +3498,6 @@
           <t>Kruk Marcin</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3606,7 +3540,6 @@
           <t>Wrzeszcz Barbara</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -3639,13 +3572,11 @@
           <t>Język polski</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
           <t>-</t>
@@ -3688,7 +3619,6 @@
           <t>Krzemińska Beata</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3731,7 +3661,6 @@
           <t>Nestoruk Lidia</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3774,7 +3703,6 @@
           <t>Marzec Renata</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3817,7 +3745,6 @@
           <t>Mucha Anna</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3860,7 +3787,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
           <t>-</t>
@@ -3903,7 +3829,6 @@
           <t>Galert Anna</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -3946,7 +3871,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr">
         <is>
           <t>-</t>
@@ -3989,7 +3913,6 @@
           <t>Misiąg Anna</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -4032,7 +3955,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
         <is>
           <t>-</t>
@@ -4075,7 +3997,6 @@
           <t>Kosin Anna</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4118,7 +4039,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4161,7 +4081,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
           <t>-</t>
@@ -4204,7 +4123,6 @@
           <t>Zając Ewa</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -4247,7 +4165,6 @@
           <t>Wójcik Kamil</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4290,7 +4207,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -4427,7 +4343,6 @@
           <t>Hudziec Agnieszka</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4564,7 +4479,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -4607,7 +4521,6 @@
           <t>Piątek-Pawłowska Bożena</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4650,7 +4563,6 @@
           <t>Wójcik Kamil</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4693,7 +4605,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4736,7 +4647,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr">
         <is>
           <t>-</t>
@@ -4826,7 +4736,6 @@
           <t>Sobczak Anna</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4869,7 +4778,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -4912,7 +4820,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
           <t>-</t>
@@ -5002,7 +4909,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5045,7 +4951,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>-</t>
@@ -5088,7 +4993,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
           <t>-</t>
@@ -5131,7 +5035,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5268,7 +5171,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr">
         <is>
           <t>-</t>
@@ -5311,7 +5213,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
           <t>-</t>
@@ -5354,7 +5255,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5397,7 +5297,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
           <t>-</t>
@@ -5487,7 +5386,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
           <t>-</t>
@@ -5530,7 +5428,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
           <t>-</t>
@@ -5573,7 +5470,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5616,7 +5512,6 @@
           <t>Nestoruk Lidia</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5706,7 +5601,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
           <t>-</t>
@@ -5749,7 +5643,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>-</t>
@@ -5792,7 +5685,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
           <t>-</t>
@@ -5835,7 +5727,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5878,7 +5769,6 @@
           <t>Hudziec Agnieszka</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5968,7 +5858,6 @@
           <t>Biczysko Wojciech</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -5998,7 +5887,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Historia</t>
+          <t>Biznes i zarządzanie</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -6008,10 +5897,9 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Kaczorowski Waldemar</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr"/>
+          <t>Smirnow-Zechman Eleonora</t>
+        </is>
+      </c>
       <c r="I127" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -6054,7 +5942,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -6097,7 +5984,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -6140,7 +6026,6 @@
           <t>Sałdyka Karolina</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
       <c r="I130" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -6371,7 +6256,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
           <t>-</t>
@@ -6461,7 +6345,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -6504,7 +6387,6 @@
           <t>Pietrycha Małgorzata</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
       <c r="I138" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -6547,7 +6429,6 @@
           <t>Taszycka Magdalena</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -6778,7 +6659,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
       <c r="I144" t="inlineStr">
         <is>
           <t>-</t>
@@ -6868,7 +6748,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
       <c r="I146" t="inlineStr">
         <is>
           <t>-</t>
@@ -6911,7 +6790,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
           <t>-</t>
@@ -6954,7 +6832,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
       <c r="I148" t="inlineStr">
         <is>
           <t>-</t>
@@ -6997,7 +6874,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr">
         <is>
           <t>-</t>
@@ -7040,7 +6916,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr">
         <is>
           <t>-</t>
@@ -7083,7 +6958,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr">
         <is>
           <t>-</t>
@@ -7126,7 +7000,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
       <c r="I152" t="inlineStr">
         <is>
           <t>-</t>
@@ -7169,7 +7042,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr">
         <is>
           <t>-</t>
@@ -7212,7 +7084,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
         <is>
           <t>-</t>
@@ -7255,7 +7126,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
         <is>
           <t>-</t>
@@ -7298,7 +7168,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr">
         <is>
           <t>-</t>
@@ -7341,7 +7210,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr">
         <is>
           <t>-</t>
@@ -7384,7 +7252,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr">
         <is>
           <t>-</t>
@@ -7427,7 +7294,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr">
         <is>
           <t>-</t>
@@ -7470,7 +7336,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr">
         <is>
           <t>-</t>
@@ -7513,7 +7378,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr">
         <is>
           <t>-</t>
@@ -7556,7 +7420,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr">
         <is>
           <t>-</t>
@@ -7599,7 +7462,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr">
         <is>
           <t>-</t>
@@ -7642,7 +7504,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr">
         <is>
           <t>-</t>
@@ -7685,7 +7546,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr">
         <is>
           <t>-</t>
@@ -7728,7 +7588,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>-</t>
@@ -7771,7 +7630,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr">
         <is>
           <t>-</t>
@@ -7814,7 +7672,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr">
         <is>
           <t>-</t>
@@ -7857,7 +7714,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>-</t>
@@ -7900,7 +7756,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
           <t>-</t>
@@ -7943,7 +7798,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr">
         <is>
           <t>-</t>
@@ -7986,7 +7840,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr">
         <is>
           <t>-</t>
@@ -8029,7 +7882,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
           <t>-</t>
@@ -8072,7 +7924,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>-</t>
@@ -8115,7 +7966,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr">
         <is>
           <t>-</t>
@@ -8158,7 +8008,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
           <t>-</t>
@@ -8201,7 +8050,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
           <t>-</t>
@@ -8244,7 +8092,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
           <t>-</t>
@@ -8287,7 +8134,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr">
         <is>
           <t>-</t>
@@ -8330,7 +8176,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr">
         <is>
           <t>-</t>
@@ -8373,7 +8218,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
       <c r="I181" t="inlineStr">
         <is>
           <t>-</t>
@@ -8416,7 +8260,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
       <c r="I182" t="inlineStr">
         <is>
           <t>-</t>
@@ -8459,7 +8302,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
       <c r="I183" t="inlineStr">
         <is>
           <t>-</t>
@@ -8502,7 +8344,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
       <c r="I184" t="inlineStr">
         <is>
           <t>-</t>
@@ -8545,7 +8386,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
       <c r="I185" t="inlineStr">
         <is>
           <t>-</t>
@@ -8588,7 +8428,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
       <c r="I186" t="inlineStr">
         <is>
           <t>-</t>
@@ -8631,7 +8470,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr">
         <is>
           <t>-</t>
@@ -8674,7 +8512,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr">
         <is>
           <t>-</t>
@@ -8717,7 +8554,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
           <t>-</t>
@@ -8760,7 +8596,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
           <t>-</t>
@@ -8803,7 +8638,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
           <t>-</t>
@@ -8846,7 +8680,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
           <t>-</t>
@@ -8889,7 +8722,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
       <c r="I193" t="inlineStr">
         <is>
           <t>-</t>
@@ -8932,7 +8764,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
           <t>-</t>
@@ -8975,7 +8806,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
       <c r="I195" t="inlineStr">
         <is>
           <t>-</t>
@@ -9018,7 +8848,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr">
         <is>
           <t>-</t>
@@ -9061,7 +8890,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr">
         <is>
           <t>-</t>
@@ -9104,7 +8932,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr">
         <is>
           <t>-</t>
@@ -9147,7 +8974,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
           <t>-</t>
@@ -9190,7 +9016,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
       <c r="I200" t="inlineStr">
         <is>
           <t>-</t>
@@ -9233,7 +9058,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
           <t>-</t>
@@ -9276,7 +9100,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
           <t>-</t>
@@ -9319,7 +9142,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
       <c r="I203" t="inlineStr">
         <is>
           <t>-</t>
@@ -9362,7 +9184,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
       <c r="I204" t="inlineStr">
         <is>
           <t>-</t>
@@ -9405,7 +9226,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
           <t>-</t>
@@ -9448,7 +9268,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
           <t>-</t>
@@ -9491,7 +9310,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
           <t>-</t>
@@ -9534,7 +9352,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
       <c r="I208" t="inlineStr">
         <is>
           <t>-</t>
@@ -9577,7 +9394,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
           <t>-</t>
@@ -9620,7 +9436,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
           <t>-</t>
@@ -9663,7 +9478,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr">
         <is>
           <t>-</t>
@@ -9706,7 +9520,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr">
         <is>
           <t>-</t>
@@ -9749,7 +9562,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
       <c r="I213" t="inlineStr">
         <is>
           <t>-</t>
@@ -9792,7 +9604,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
           <t>-</t>
@@ -9835,7 +9646,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
           <t>-</t>
@@ -9878,7 +9688,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
           <t>-</t>
@@ -9921,7 +9730,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
       <c r="I217" t="inlineStr">
         <is>
           <t>-</t>
@@ -9964,7 +9772,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
       <c r="I218" t="inlineStr">
         <is>
           <t>-</t>
@@ -10007,7 +9814,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
       <c r="I219" t="inlineStr">
         <is>
           <t>-</t>
@@ -10050,7 +9856,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
       <c r="I220" t="inlineStr">
         <is>
           <t>-</t>
@@ -10093,7 +9898,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
       <c r="I221" t="inlineStr">
         <is>
           <t>-</t>
@@ -10136,7 +9940,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
       <c r="I222" t="inlineStr">
         <is>
           <t>-</t>
@@ -10179,7 +9982,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
       <c r="I223" t="inlineStr">
         <is>
           <t>-</t>
@@ -10222,7 +10024,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
       <c r="I224" t="inlineStr">
         <is>
           <t>-</t>
@@ -10265,7 +10066,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
       <c r="I225" t="inlineStr">
         <is>
           <t>-</t>
@@ -10308,7 +10108,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
       <c r="I226" t="inlineStr">
         <is>
           <t>-</t>
@@ -10351,7 +10150,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
       <c r="I227" t="inlineStr">
         <is>
           <t>-</t>
@@ -10394,7 +10192,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
       <c r="I228" t="inlineStr">
         <is>
           <t>-</t>
@@ -10437,7 +10234,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
       <c r="I229" t="inlineStr">
         <is>
           <t>-</t>
@@ -10480,7 +10276,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
       <c r="I230" t="inlineStr">
         <is>
           <t>-</t>
@@ -10523,7 +10318,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr">
         <is>
           <t>-</t>
@@ -10566,7 +10360,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
       <c r="I232" t="inlineStr">
         <is>
           <t>-</t>
@@ -10609,7 +10402,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
       <c r="I233" t="inlineStr">
         <is>
           <t>-</t>
@@ -10652,7 +10444,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
       <c r="I234" t="inlineStr">
         <is>
           <t>-</t>
@@ -10695,7 +10486,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
       <c r="I235" t="inlineStr">
         <is>
           <t>-</t>
@@ -10738,7 +10528,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
       <c r="I236" t="inlineStr">
         <is>
           <t>-</t>
@@ -10781,7 +10570,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
       <c r="I237" t="inlineStr">
         <is>
           <t>-</t>
@@ -10824,7 +10612,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
       <c r="I238" t="inlineStr">
         <is>
           <t>-</t>
@@ -10867,7 +10654,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
       <c r="I239" t="inlineStr">
         <is>
           <t>-</t>
@@ -10910,7 +10696,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
       <c r="I240" t="inlineStr">
         <is>
           <t>-</t>
@@ -10953,7 +10738,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
       <c r="I241" t="inlineStr">
         <is>
           <t>-</t>
@@ -10996,7 +10780,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
       <c r="I242" t="inlineStr">
         <is>
           <t>-</t>
@@ -11039,7 +10822,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
       <c r="I243" t="inlineStr">
         <is>
           <t>-</t>
@@ -11082,7 +10864,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
       <c r="I244" t="inlineStr">
         <is>
           <t>-</t>
@@ -11125,7 +10906,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
       <c r="I245" t="inlineStr">
         <is>
           <t>-</t>
@@ -11168,7 +10948,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
       <c r="I246" t="inlineStr">
         <is>
           <t>-</t>
@@ -11211,7 +10990,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
           <t>-</t>
@@ -11254,7 +11032,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
       <c r="I248" t="inlineStr">
         <is>
           <t>-</t>
@@ -11297,7 +11074,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
       <c r="I249" t="inlineStr">
         <is>
           <t>-</t>
@@ -11340,7 +11116,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
       <c r="I250" t="inlineStr">
         <is>
           <t>-</t>
@@ -11383,7 +11158,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
       <c r="I251" t="inlineStr">
         <is>
           <t>-</t>
@@ -11426,7 +11200,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
       <c r="I252" t="inlineStr">
         <is>
           <t>-</t>
@@ -11469,7 +11242,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
       <c r="I253" t="inlineStr">
         <is>
           <t>-</t>
@@ -11512,7 +11284,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
       <c r="I254" t="inlineStr">
         <is>
           <t>-</t>
@@ -11555,7 +11326,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr">
         <is>
           <t>-</t>
@@ -11598,7 +11368,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
       <c r="I256" t="inlineStr">
         <is>
           <t>-</t>
@@ -11641,7 +11410,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
       <c r="I257" t="inlineStr">
         <is>
           <t>-</t>
@@ -11684,7 +11452,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
       <c r="I258" t="inlineStr">
         <is>
           <t>-</t>
@@ -11727,7 +11494,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr">
         <is>
           <t>-</t>
@@ -11770,7 +11536,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
       <c r="I260" t="inlineStr">
         <is>
           <t>-</t>
@@ -11813,7 +11578,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
       <c r="I261" t="inlineStr">
         <is>
           <t>-</t>
@@ -11856,7 +11620,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
       <c r="I262" t="inlineStr">
         <is>
           <t>-</t>
@@ -11899,7 +11662,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
       <c r="I263" t="inlineStr">
         <is>
           <t>-</t>
@@ -11942,7 +11704,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
       <c r="I264" t="inlineStr">
         <is>
           <t>-</t>
@@ -11985,7 +11746,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
       <c r="I265" t="inlineStr">
         <is>
           <t>-</t>
@@ -12028,7 +11788,6 @@
           <t>Rejno Julita</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
       <c r="I266" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12165,7 +11924,6 @@
           <t>Rejno Julita</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
       <c r="I269" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12302,7 +12060,6 @@
           <t>Rejno Julita</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
       <c r="I272" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12345,7 +12102,6 @@
           <t>Jastrzębska-Majtyka Agnieszka</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
       <c r="I273" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -12388,7 +12144,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
       <c r="I274" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12431,7 +12186,6 @@
           <t>Filipiak Wiesław</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
       <c r="I275" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12474,7 +12228,6 @@
           <t>Rejno Julita</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
       <c r="I276" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12517,7 +12270,6 @@
           <t>Jastrzębska-Majtyka Agnieszka</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr"/>
       <c r="I277" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -12560,7 +12312,6 @@
           <t>Kończyńska Małgorzata</t>
         </is>
       </c>
-      <c r="H278" t="inlineStr"/>
       <c r="I278" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12603,7 +12354,6 @@
           <t>Filipiak Wiesław</t>
         </is>
       </c>
-      <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12646,7 +12396,6 @@
           <t>Rejno Julita</t>
         </is>
       </c>
-      <c r="H280" t="inlineStr"/>
       <c r="I280" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12689,7 +12438,6 @@
           <t>Jastrzębska-Majtyka Agnieszka</t>
         </is>
       </c>
-      <c r="H281" t="inlineStr"/>
       <c r="I281" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -12732,7 +12480,6 @@
           <t>Rejno Julita</t>
         </is>
       </c>
-      <c r="H282" t="inlineStr"/>
       <c r="I282" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12775,7 +12522,6 @@
           <t>Jastrzębska-Majtyka Agnieszka</t>
         </is>
       </c>
-      <c r="H283" t="inlineStr"/>
       <c r="I283" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -12818,7 +12564,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H284" t="inlineStr"/>
       <c r="I284" t="inlineStr">
         <is>
           <t>-</t>
@@ -12861,7 +12606,6 @@
           <t>Jastrzębska-Majtyka Agnieszka</t>
         </is>
       </c>
-      <c r="H285" t="inlineStr"/>
       <c r="I285" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -12904,7 +12648,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H286" t="inlineStr"/>
       <c r="I286" t="inlineStr">
         <is>
           <t>-</t>
@@ -12947,7 +12690,6 @@
           <t>Krzemińska Beata</t>
         </is>
       </c>
-      <c r="H287" t="inlineStr"/>
       <c r="I287" t="inlineStr">
         <is>
           <t>Dodatkowo płatne</t>
@@ -12990,7 +12732,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H288" t="inlineStr"/>
       <c r="I288" t="inlineStr">
         <is>
           <t>-</t>
@@ -13033,7 +12774,6 @@
           <t>Jastrzębska-Majtyka Agnieszka</t>
         </is>
       </c>
-      <c r="H289" t="inlineStr"/>
       <c r="I289" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -13076,7 +12816,6 @@
           <t>Uczniowie przychodzą później</t>
         </is>
       </c>
-      <c r="H290" t="inlineStr"/>
       <c r="I290" t="inlineStr">
         <is>
           <t>-</t>
@@ -13119,7 +12858,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H291" t="inlineStr"/>
       <c r="I291" t="inlineStr">
         <is>
           <t>-</t>
@@ -13162,7 +12900,6 @@
           <t>Jastrzębska-Majtyka Agnieszka</t>
         </is>
       </c>
-      <c r="H292" t="inlineStr"/>
       <c r="I292" t="inlineStr">
         <is>
           <t>Bezpłatne</t>
@@ -13205,7 +12942,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr"/>
       <c r="I293" t="inlineStr">
         <is>
           <t>-</t>
@@ -13248,7 +12984,6 @@
           <t>Uczniowie zwolnieni do domu</t>
         </is>
       </c>
-      <c r="H294" t="inlineStr"/>
       <c r="I294" t="inlineStr">
         <is>
           <t>-</t>
@@ -13291,7 +13026,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H295" t="inlineStr"/>
       <c r="I295" t="inlineStr">
         <is>
           <t>-</t>
@@ -13334,7 +13068,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H296" t="inlineStr"/>
       <c r="I296" t="inlineStr">
         <is>
           <t>-</t>
@@ -13377,7 +13110,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H297" t="inlineStr"/>
       <c r="I297" t="inlineStr">
         <is>
           <t>-</t>
@@ -13420,7 +13152,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H298" t="inlineStr"/>
       <c r="I298" t="inlineStr">
         <is>
           <t>-</t>
@@ -13463,7 +13194,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H299" t="inlineStr"/>
       <c r="I299" t="inlineStr">
         <is>
           <t>-</t>
@@ -13506,7 +13236,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H300" t="inlineStr"/>
       <c r="I300" t="inlineStr">
         <is>
           <t>-</t>
@@ -13549,7 +13278,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H301" t="inlineStr"/>
       <c r="I301" t="inlineStr">
         <is>
           <t>-</t>
@@ -13592,7 +13320,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H302" t="inlineStr"/>
       <c r="I302" t="inlineStr">
         <is>
           <t>-</t>
@@ -13635,7 +13362,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H303" t="inlineStr"/>
       <c r="I303" t="inlineStr">
         <is>
           <t>-</t>
@@ -13678,7 +13404,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H304" t="inlineStr"/>
       <c r="I304" t="inlineStr">
         <is>
           <t>-</t>
@@ -13721,7 +13446,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H305" t="inlineStr"/>
       <c r="I305" t="inlineStr">
         <is>
           <t>-</t>
@@ -13764,7 +13488,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H306" t="inlineStr"/>
       <c r="I306" t="inlineStr">
         <is>
           <t>-</t>
@@ -13807,7 +13530,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H307" t="inlineStr"/>
       <c r="I307" t="inlineStr">
         <is>
           <t>-</t>
@@ -13850,7 +13572,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H308" t="inlineStr"/>
       <c r="I308" t="inlineStr">
         <is>
           <t>-</t>
@@ -13893,7 +13614,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H309" t="inlineStr"/>
       <c r="I309" t="inlineStr">
         <is>
           <t>-</t>
@@ -13936,7 +13656,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H310" t="inlineStr"/>
       <c r="I310" t="inlineStr">
         <is>
           <t>-</t>
@@ -13979,7 +13698,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H311" t="inlineStr"/>
       <c r="I311" t="inlineStr">
         <is>
           <t>-</t>
@@ -14022,7 +13740,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H312" t="inlineStr"/>
       <c r="I312" t="inlineStr">
         <is>
           <t>-</t>
@@ -14065,7 +13782,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H313" t="inlineStr"/>
       <c r="I313" t="inlineStr">
         <is>
           <t>-</t>
@@ -14108,7 +13824,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H314" t="inlineStr"/>
       <c r="I314" t="inlineStr">
         <is>
           <t>-</t>
@@ -14151,7 +13866,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H315" t="inlineStr"/>
       <c r="I315" t="inlineStr">
         <is>
           <t>-</t>
@@ -14194,7 +13908,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H316" t="inlineStr"/>
       <c r="I316" t="inlineStr">
         <is>
           <t>-</t>
@@ -14237,7 +13950,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H317" t="inlineStr"/>
       <c r="I317" t="inlineStr">
         <is>
           <t>-</t>
@@ -14280,7 +13992,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H318" t="inlineStr"/>
       <c r="I318" t="inlineStr">
         <is>
           <t>-</t>
@@ -14323,7 +14034,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H319" t="inlineStr"/>
       <c r="I319" t="inlineStr">
         <is>
           <t>-</t>
@@ -14366,7 +14076,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H320" t="inlineStr"/>
       <c r="I320" t="inlineStr">
         <is>
           <t>-</t>
@@ -14409,7 +14118,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H321" t="inlineStr"/>
       <c r="I321" t="inlineStr">
         <is>
           <t>-</t>
@@ -14452,7 +14160,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H322" t="inlineStr"/>
       <c r="I322" t="inlineStr">
         <is>
           <t>-</t>
@@ -14495,7 +14202,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H323" t="inlineStr"/>
       <c r="I323" t="inlineStr">
         <is>
           <t>-</t>
@@ -14538,7 +14244,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H324" t="inlineStr"/>
       <c r="I324" t="inlineStr">
         <is>
           <t>-</t>
@@ -14581,7 +14286,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H325" t="inlineStr"/>
       <c r="I325" t="inlineStr">
         <is>
           <t>-</t>
@@ -14624,7 +14328,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H326" t="inlineStr"/>
       <c r="I326" t="inlineStr">
         <is>
           <t>-</t>
@@ -14667,7 +14370,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H327" t="inlineStr"/>
       <c r="I327" t="inlineStr">
         <is>
           <t>-</t>
@@ -14710,7 +14412,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr"/>
       <c r="I328" t="inlineStr">
         <is>
           <t>-</t>
@@ -14753,7 +14454,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H329" t="inlineStr"/>
       <c r="I329" t="inlineStr">
         <is>
           <t>-</t>
@@ -14796,7 +14496,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H330" t="inlineStr"/>
       <c r="I330" t="inlineStr">
         <is>
           <t>-</t>
@@ -14839,7 +14538,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H331" t="inlineStr"/>
       <c r="I331" t="inlineStr">
         <is>
           <t>-</t>
@@ -14882,7 +14580,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H332" t="inlineStr"/>
       <c r="I332" t="inlineStr">
         <is>
           <t>-</t>
@@ -14925,7 +14622,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H333" t="inlineStr"/>
       <c r="I333" t="inlineStr">
         <is>
           <t>-</t>
@@ -14968,7 +14664,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H334" t="inlineStr"/>
       <c r="I334" t="inlineStr">
         <is>
           <t>-</t>
@@ -15011,7 +14706,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H335" t="inlineStr"/>
       <c r="I335" t="inlineStr">
         <is>
           <t>-</t>
@@ -15054,7 +14748,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H336" t="inlineStr"/>
       <c r="I336" t="inlineStr">
         <is>
           <t>-</t>
@@ -15097,7 +14790,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H337" t="inlineStr"/>
       <c r="I337" t="inlineStr">
         <is>
           <t>-</t>
@@ -15140,7 +14832,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H338" t="inlineStr"/>
       <c r="I338" t="inlineStr">
         <is>
           <t>-</t>
@@ -15183,7 +14874,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H339" t="inlineStr"/>
       <c r="I339" t="inlineStr">
         <is>
           <t>-</t>
@@ -15226,7 +14916,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H340" t="inlineStr"/>
       <c r="I340" t="inlineStr">
         <is>
           <t>-</t>
@@ -15269,7 +14958,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H341" t="inlineStr"/>
       <c r="I341" t="inlineStr">
         <is>
           <t>-</t>
@@ -15312,7 +15000,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H342" t="inlineStr"/>
       <c r="I342" t="inlineStr">
         <is>
           <t>-</t>
@@ -15355,7 +15042,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H343" t="inlineStr"/>
       <c r="I343" t="inlineStr">
         <is>
           <t>-</t>
@@ -15398,7 +15084,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H344" t="inlineStr"/>
       <c r="I344" t="inlineStr">
         <is>
           <t>-</t>
@@ -15441,7 +15126,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H345" t="inlineStr"/>
       <c r="I345" t="inlineStr">
         <is>
           <t>-</t>
@@ -15484,7 +15168,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H346" t="inlineStr"/>
       <c r="I346" t="inlineStr">
         <is>
           <t>-</t>
@@ -15527,7 +15210,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H347" t="inlineStr"/>
       <c r="I347" t="inlineStr">
         <is>
           <t>-</t>
@@ -15570,7 +15252,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H348" t="inlineStr"/>
       <c r="I348" t="inlineStr">
         <is>
           <t>-</t>
@@ -15613,7 +15294,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H349" t="inlineStr"/>
       <c r="I349" t="inlineStr">
         <is>
           <t>-</t>
@@ -15656,7 +15336,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H350" t="inlineStr"/>
       <c r="I350" t="inlineStr">
         <is>
           <t>-</t>
@@ -15699,7 +15378,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H351" t="inlineStr"/>
       <c r="I351" t="inlineStr">
         <is>
           <t>-</t>
@@ -15742,7 +15420,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H352" t="inlineStr"/>
       <c r="I352" t="inlineStr">
         <is>
           <t>-</t>
@@ -15785,7 +15462,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H353" t="inlineStr"/>
       <c r="I353" t="inlineStr">
         <is>
           <t>-</t>
@@ -15828,7 +15504,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H354" t="inlineStr"/>
       <c r="I354" t="inlineStr">
         <is>
           <t>-</t>
@@ -15871,7 +15546,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H355" t="inlineStr"/>
       <c r="I355" t="inlineStr">
         <is>
           <t>-</t>
@@ -15914,7 +15588,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H356" t="inlineStr"/>
       <c r="I356" t="inlineStr">
         <is>
           <t>-</t>
@@ -15957,7 +15630,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H357" t="inlineStr"/>
       <c r="I357" t="inlineStr">
         <is>
           <t>-</t>
@@ -16000,7 +15672,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr"/>
       <c r="I358" t="inlineStr">
         <is>
           <t>-</t>
@@ -16117,7 +15788,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>-</t>
@@ -16160,7 +15830,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>-</t>
@@ -16203,7 +15872,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>-</t>
@@ -16236,13 +15904,11 @@
           <t>język polski</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>-</t>
@@ -16285,7 +15951,6 @@
           <t>Zastępstwo</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>-</t>
@@ -16374,7 +16039,6 @@
           <t>Ostrowska Ewa</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -16402,7 +16066,6 @@
           <t>Kosin Anna</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -16430,7 +16093,6 @@
           <t>Małecka Barbara</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -16458,7 +16120,6 @@
           <t>Mucha Anna</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -16486,7 +16147,6 @@
           <t>Skarupa Agnieszka</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -16514,7 +16174,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -16542,7 +16201,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -16570,7 +16228,6 @@
           <t>Misiąg Anna</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -16598,7 +16255,6 @@
           <t>Ulanowska Magdalena</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -16626,7 +16282,6 @@
           <t>Socha Dariusz</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -16654,7 +16309,6 @@
           <t>Cieśla Marcin</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -16682,7 +16336,6 @@
           <t>Małecka Barbara</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -16710,7 +16363,6 @@
           <t>Kruk Marcin</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" t="inlineStr">
@@ -16738,7 +16390,6 @@
           <t>Krycia Ewelina</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" t="inlineStr">
@@ -16766,7 +16417,6 @@
           <t>Danielewski Paweł</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -16794,7 +16444,6 @@
           <t>Skarupa Agnieszka</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -16822,7 +16471,6 @@
           <t>Zaleska Magdalena</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" t="inlineStr">
@@ -16850,7 +16498,6 @@
           <t>Krzemińska Beata</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" t="inlineStr">
@@ -16878,7 +16525,6 @@
           <t>Płatek Krzysztof</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -16906,7 +16552,6 @@
           <t>Smirnow-Zechman Eleonora</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" t="inlineStr">
@@ -16934,7 +16579,6 @@
           <t>Najwer Maciej</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" t="inlineStr">
@@ -16962,7 +16606,6 @@
           <t>Danielewski Paweł</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" t="inlineStr">
@@ -16990,7 +16633,6 @@
           <t>Leńczowska Iwona</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" t="inlineStr">
@@ -17018,7 +16660,6 @@
           <t>Smereka Alicja</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" t="inlineStr">
@@ -17046,7 +16687,6 @@
           <t>Taszycka Magdalena</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" t="inlineStr">
@@ -17106,7 +16746,6 @@
           <t>Krycia Ewelina</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" t="inlineStr">
@@ -17134,7 +16773,6 @@
           <t>Karczmarz Aleksandra</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" t="inlineStr">
@@ -17162,7 +16800,6 @@
           <t>Misiąg Anna</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" t="inlineStr">
@@ -17190,7 +16827,6 @@
           <t>Dalach Krystyna</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" t="inlineStr">
@@ -17218,7 +16854,6 @@
           <t>Wojciechowski Łukasz</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" t="inlineStr">
@@ -17246,7 +16881,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" t="inlineStr">
@@ -17274,7 +16908,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" t="inlineStr">
@@ -17302,7 +16935,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" t="inlineStr">
@@ -17330,7 +16962,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" t="inlineStr">
@@ -17358,7 +16989,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" t="inlineStr">
@@ -17386,7 +17016,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" t="inlineStr">
@@ -17414,7 +17043,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" t="inlineStr">
@@ -17442,7 +17070,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" t="inlineStr">
@@ -17470,7 +17097,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" t="inlineStr">
@@ -17498,7 +17124,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" t="inlineStr">
@@ -17526,7 +17151,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" t="inlineStr">
@@ -17554,7 +17178,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" t="inlineStr">
@@ -17582,7 +17205,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" t="inlineStr">
@@ -17610,7 +17232,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" t="inlineStr">
@@ -17638,7 +17259,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" t="inlineStr">
@@ -17666,7 +17286,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" t="inlineStr">
@@ -17694,7 +17313,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" t="inlineStr">
@@ -17722,7 +17340,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" t="inlineStr">
@@ -17750,7 +17367,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" t="inlineStr">
@@ -17778,7 +17394,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" t="inlineStr">
@@ -17806,7 +17421,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" t="inlineStr">
@@ -17834,7 +17448,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" t="inlineStr">
@@ -17862,7 +17475,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" t="inlineStr">
@@ -17890,7 +17502,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" t="inlineStr">
@@ -17918,7 +17529,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>

</xml_diff>